<commit_message>
Saving Progress after paper searching and arranging year wise
</commit_message>
<xml_diff>
--- a/Attainment Calculation/Attainment  Calculation Barate Batch/CR3_22317 - Data Structures Using _C_ (1).xlsx
+++ b/Attainment Calculation/Attainment  Calculation Barate Batch/CR3_22317 - Data Structures Using _C_ (1).xlsx
@@ -1,16 +1,10 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27928"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="7" rupBuild="9303"/>
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MSBTE-28\Documents\ada\gpd_nba\Attainment Calculation\Atainment Calculation Barate Batch\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D8BE564-DF94-4E10-8443-5AFB68EA5570}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="21840" windowHeight="13740" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="PO Set Target attain level" sheetId="1" r:id="rId1"/>
@@ -45,12 +39,12 @@
 </file>
 
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author/>
   </authors>
   <commentList>
-    <comment ref="D12" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000001000000}">
+    <comment ref="D12" authorId="0">
       <text>
         <r>
           <rPr>
@@ -1159,7 +1153,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
@@ -3209,20 +3203,61 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="2" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="43" fillId="0" borderId="92" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="42" fillId="0" borderId="92" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="43" fillId="0" borderId="93" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="42" fillId="0" borderId="93" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="93" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="93" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="93" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="93" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="93" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="93" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="9" fillId="5" borderId="93" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="44" fillId="2" borderId="93" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="93" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="93" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="93" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="93" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -3232,87 +3267,27 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="10" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="16" fillId="11" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="7" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="4" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="2" fontId="4" fillId="4" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="4" borderId="46" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="47" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="4" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="8" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="9" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="12" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="16" fillId="13" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -3333,15 +3308,40 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="46" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="47" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="16" fillId="4" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -3350,16 +3350,49 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
+    <xf numFmtId="0" fontId="16" fillId="10" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="16" fillId="11" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="7" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="4" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="8" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="9" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="46" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="66" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="28" fillId="4" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="55" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="57" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -3372,32 +3405,11 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="65" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="46" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="66" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="2" fontId="28" fillId="4" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="55" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="4" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="70" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="64" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="46" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -3408,6 +3420,36 @@
     <xf numFmtId="0" fontId="30" fillId="4" borderId="67" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="21" fillId="4" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="70" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="64" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="75" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="54" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="76" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -3425,28 +3467,38 @@
     <xf numFmtId="0" fontId="4" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="75" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="54" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="76" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="12" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="38" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="64" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="15" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="34" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -3467,40 +3519,25 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="64" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="38" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="64" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="38" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="35" fillId="4" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="3" fillId="4" borderId="46" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="15" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="82" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="84" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="54" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="83" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="85" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="64" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="54" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="36" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="46" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -3524,71 +3561,28 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="64" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="82" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="84" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="54" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="83" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="85" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="64" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="38" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="54" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="4" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="3" fillId="4" borderId="46" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="43" fillId="0" borderId="92" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="42" fillId="0" borderId="92" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="43" fillId="0" borderId="93" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="42" fillId="0" borderId="93" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="93" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="93" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="93" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="93" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="93" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="93" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="93" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="93" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="93" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="93" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="9" fillId="5" borderId="93" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="44" fillId="2" borderId="93" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -3623,7 +3617,7 @@
         <xdr:cNvPr id="3" name="Shape 3">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000003000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-000003000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -3687,7 +3681,7 @@
         <xdr:cNvPr id="4" name="Shape 4">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000004000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-000004000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -3751,7 +3745,7 @@
         <xdr:cNvPr id="2" name="Shape 3">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-000002000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -3815,7 +3809,7 @@
         <xdr:cNvPr id="5" name="Shape 3">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000005000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-000005000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -3879,7 +3873,7 @@
         <xdr:cNvPr id="6" name="Shape 4">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000006000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-000006000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -3948,7 +3942,7 @@
         <xdr:cNvPr id="5" name="Shape 5">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0200-000005000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0200-000005000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -4019,7 +4013,7 @@
         <xdr:cNvPr id="6" name="Shape 6">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0300-000006000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0300-000006000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -4272,7 +4266,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <tabColor rgb="FFFFFF00"/>
   </sheetPr>
@@ -4309,10 +4303,10 @@
       <c r="C3" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="D3" s="215" t="s">
+      <c r="D3" s="205" t="s">
         <v>2</v>
       </c>
-      <c r="E3" s="210"/>
+      <c r="E3" s="206"/>
       <c r="F3" s="4"/>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.25">
@@ -4321,10 +4315,10 @@
       <c r="C4" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="D4" s="215">
+      <c r="D4" s="205">
         <v>22317</v>
       </c>
-      <c r="E4" s="210"/>
+      <c r="E4" s="206"/>
       <c r="F4" s="4"/>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.25">
@@ -4333,10 +4327,10 @@
       <c r="C5" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="D5" s="215" t="s">
+      <c r="D5" s="205" t="s">
         <v>5</v>
       </c>
-      <c r="E5" s="210"/>
+      <c r="E5" s="206"/>
       <c r="F5" s="4"/>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.25">
@@ -4345,10 +4339,10 @@
       <c r="C6" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="D6" s="215" t="s">
+      <c r="D6" s="205" t="s">
         <v>7</v>
       </c>
-      <c r="E6" s="210"/>
+      <c r="E6" s="206"/>
       <c r="F6" s="4"/>
     </row>
     <row r="7" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
@@ -4470,390 +4464,390 @@
       <c r="M16" s="4"/>
     </row>
     <row r="17" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="B17" s="333" t="s">
+      <c r="B17" s="210" t="s">
         <v>20</v>
       </c>
-      <c r="C17" s="333" t="s">
+      <c r="C17" s="210" t="s">
         <v>21</v>
       </c>
-      <c r="D17" s="334"/>
-      <c r="E17" s="333" t="s">
+      <c r="D17" s="211"/>
+      <c r="E17" s="210" t="s">
         <v>22</v>
       </c>
-      <c r="F17" s="334"/>
-      <c r="G17" s="334"/>
-      <c r="H17" s="334"/>
-      <c r="I17" s="334"/>
-      <c r="J17" s="334"/>
-      <c r="K17" s="334"/>
-      <c r="L17" s="333" t="s">
+      <c r="F17" s="211"/>
+      <c r="G17" s="211"/>
+      <c r="H17" s="211"/>
+      <c r="I17" s="211"/>
+      <c r="J17" s="211"/>
+      <c r="K17" s="211"/>
+      <c r="L17" s="210" t="s">
         <v>23</v>
       </c>
-      <c r="M17" s="334"/>
+      <c r="M17" s="211"/>
     </row>
     <row r="18" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="B18" s="334"/>
-      <c r="C18" s="334"/>
-      <c r="D18" s="334"/>
-      <c r="E18" s="335" t="s">
+      <c r="B18" s="211"/>
+      <c r="C18" s="211"/>
+      <c r="D18" s="211"/>
+      <c r="E18" s="197" t="s">
         <v>24</v>
       </c>
-      <c r="F18" s="335" t="s">
+      <c r="F18" s="197" t="s">
         <v>25</v>
       </c>
-      <c r="G18" s="335" t="s">
+      <c r="G18" s="197" t="s">
         <v>26</v>
       </c>
-      <c r="H18" s="335" t="s">
+      <c r="H18" s="197" t="s">
         <v>27</v>
       </c>
-      <c r="I18" s="335" t="s">
+      <c r="I18" s="197" t="s">
         <v>28</v>
       </c>
-      <c r="J18" s="335" t="s">
+      <c r="J18" s="197" t="s">
         <v>29</v>
       </c>
-      <c r="K18" s="335" t="s">
+      <c r="K18" s="197" t="s">
         <v>30</v>
       </c>
-      <c r="L18" s="335" t="s">
+      <c r="L18" s="197" t="s">
         <v>31</v>
       </c>
-      <c r="M18" s="335" t="s">
+      <c r="M18" s="197" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="19" spans="1:25" ht="122.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B19" s="334"/>
-      <c r="C19" s="334"/>
-      <c r="D19" s="334"/>
-      <c r="E19" s="336" t="s">
+      <c r="B19" s="211"/>
+      <c r="C19" s="211"/>
+      <c r="D19" s="211"/>
+      <c r="E19" s="198" t="s">
         <v>33</v>
       </c>
-      <c r="F19" s="336" t="s">
+      <c r="F19" s="198" t="s">
         <v>34</v>
       </c>
-      <c r="G19" s="336" t="s">
+      <c r="G19" s="198" t="s">
         <v>35</v>
       </c>
-      <c r="H19" s="336" t="s">
+      <c r="H19" s="198" t="s">
         <v>36</v>
       </c>
-      <c r="I19" s="336" t="s">
+      <c r="I19" s="198" t="s">
         <v>37</v>
       </c>
-      <c r="J19" s="336" t="s">
+      <c r="J19" s="198" t="s">
         <v>38</v>
       </c>
-      <c r="K19" s="336" t="s">
+      <c r="K19" s="198" t="s">
         <v>39</v>
       </c>
-      <c r="L19" s="336" t="s">
+      <c r="L19" s="198" t="s">
         <v>40</v>
       </c>
-      <c r="M19" s="336" t="s">
+      <c r="M19" s="198" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="20" spans="1:25" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B20" s="337">
+      <c r="B20" s="199">
         <v>1</v>
       </c>
-      <c r="C20" s="337" t="str">
+      <c r="C20" s="199" t="str">
         <f t="shared" ref="C20:D20" si="0">C8</f>
         <v>CO1</v>
       </c>
-      <c r="D20" s="335" t="str">
+      <c r="D20" s="197" t="str">
         <f t="shared" si="0"/>
         <v>Perform basic operations on arrays</v>
       </c>
-      <c r="E20" s="344">
+      <c r="E20" s="204">
         <v>3</v>
       </c>
-      <c r="F20" s="344">
+      <c r="F20" s="204">
         <v>2</v>
       </c>
-      <c r="G20" s="344">
+      <c r="G20" s="204">
         <v>2</v>
       </c>
-      <c r="H20" s="344">
+      <c r="H20" s="204">
         <v>1</v>
       </c>
-      <c r="I20" s="344" t="s">
+      <c r="I20" s="204" t="s">
         <v>252</v>
       </c>
-      <c r="J20" s="344" t="s">
+      <c r="J20" s="204" t="s">
         <v>252</v>
       </c>
-      <c r="K20" s="344" t="s">
+      <c r="K20" s="204" t="s">
         <v>252</v>
       </c>
-      <c r="L20" s="344">
+      <c r="L20" s="204">
         <v>3</v>
       </c>
-      <c r="M20" s="344">
+      <c r="M20" s="204">
         <v>2</v>
       </c>
     </row>
     <row r="21" spans="1:25" ht="24" x14ac:dyDescent="0.25">
-      <c r="B21" s="337">
+      <c r="B21" s="199">
         <v>2</v>
       </c>
-      <c r="C21" s="337" t="str">
+      <c r="C21" s="199" t="str">
         <f t="shared" ref="C21:D21" si="1">C9</f>
         <v>CO2</v>
       </c>
-      <c r="D21" s="335" t="str">
+      <c r="D21" s="197" t="str">
         <f t="shared" si="1"/>
         <v>Apply different searching and sorting techniques.</v>
       </c>
-      <c r="E21" s="344">
+      <c r="E21" s="204">
         <v>3</v>
       </c>
-      <c r="F21" s="344">
+      <c r="F21" s="204">
         <v>3</v>
       </c>
-      <c r="G21" s="344">
+      <c r="G21" s="204">
         <v>2</v>
       </c>
-      <c r="H21" s="344">
+      <c r="H21" s="204">
         <v>2</v>
       </c>
-      <c r="I21" s="344" t="s">
+      <c r="I21" s="204" t="s">
         <v>252</v>
       </c>
-      <c r="J21" s="344" t="s">
+      <c r="J21" s="204" t="s">
         <v>252</v>
       </c>
-      <c r="K21" s="344">
+      <c r="K21" s="204">
         <v>1</v>
       </c>
-      <c r="L21" s="344">
+      <c r="L21" s="204">
         <v>3</v>
       </c>
-      <c r="M21" s="344">
+      <c r="M21" s="204">
         <v>2</v>
       </c>
     </row>
     <row r="22" spans="1:25" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B22" s="337">
+      <c r="B22" s="199">
         <v>3</v>
       </c>
-      <c r="C22" s="337" t="str">
+      <c r="C22" s="199" t="str">
         <f t="shared" ref="C22:D22" si="2">C10</f>
         <v>CO3</v>
       </c>
-      <c r="D22" s="335" t="str">
+      <c r="D22" s="197" t="str">
         <f t="shared" si="2"/>
         <v>Implement basic operations on stack and queue using array representation</v>
       </c>
-      <c r="E22" s="344">
+      <c r="E22" s="204">
         <v>3</v>
       </c>
-      <c r="F22" s="344">
+      <c r="F22" s="204">
         <v>2</v>
       </c>
-      <c r="G22" s="344">
+      <c r="G22" s="204">
         <v>3</v>
       </c>
-      <c r="H22" s="344">
+      <c r="H22" s="204">
         <v>2</v>
       </c>
-      <c r="I22" s="344" t="s">
+      <c r="I22" s="204" t="s">
         <v>252</v>
       </c>
-      <c r="J22" s="344" t="s">
+      <c r="J22" s="204" t="s">
         <v>252</v>
       </c>
-      <c r="K22" s="344" t="s">
+      <c r="K22" s="204" t="s">
         <v>252</v>
       </c>
-      <c r="L22" s="344">
+      <c r="L22" s="204">
         <v>3</v>
       </c>
-      <c r="M22" s="344">
+      <c r="M22" s="204">
         <v>2</v>
       </c>
     </row>
     <row r="23" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B23" s="337">
+      <c r="B23" s="199">
         <v>4</v>
       </c>
-      <c r="C23" s="337" t="str">
+      <c r="C23" s="199" t="str">
         <f t="shared" ref="C23:D23" si="3">C11</f>
         <v>CO4</v>
       </c>
-      <c r="D23" s="335" t="str">
+      <c r="D23" s="197" t="str">
         <f t="shared" si="3"/>
         <v xml:space="preserve"> Implement basic operations on Linked List</v>
       </c>
-      <c r="E23" s="344">
+      <c r="E23" s="204">
         <v>3</v>
       </c>
-      <c r="F23" s="344">
+      <c r="F23" s="204">
         <v>2</v>
       </c>
-      <c r="G23" s="344">
+      <c r="G23" s="204">
         <v>3</v>
       </c>
-      <c r="H23" s="344">
+      <c r="H23" s="204">
         <v>2</v>
       </c>
-      <c r="I23" s="344" t="s">
+      <c r="I23" s="204" t="s">
         <v>252</v>
       </c>
-      <c r="J23" s="344" t="s">
+      <c r="J23" s="204" t="s">
         <v>252</v>
       </c>
-      <c r="K23" s="344" t="s">
+      <c r="K23" s="204" t="s">
         <v>252</v>
       </c>
-      <c r="L23" s="344">
+      <c r="L23" s="204">
         <v>3</v>
       </c>
-      <c r="M23" s="344">
+      <c r="M23" s="204">
         <v>2</v>
       </c>
     </row>
     <row r="24" spans="1:25" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B24" s="337">
+      <c r="B24" s="199">
         <v>5</v>
       </c>
-      <c r="C24" s="337" t="str">
+      <c r="C24" s="199" t="str">
         <f t="shared" ref="C24:D24" si="4">C12</f>
         <v>CO5</v>
       </c>
-      <c r="D24" s="335" t="str">
+      <c r="D24" s="197" t="str">
         <f t="shared" si="4"/>
         <v>Implement program to create and traverse tree to solve problems</v>
       </c>
-      <c r="E24" s="344">
+      <c r="E24" s="204">
         <v>3</v>
       </c>
-      <c r="F24" s="344">
+      <c r="F24" s="204">
         <v>3</v>
       </c>
-      <c r="G24" s="344">
+      <c r="G24" s="204">
         <v>3</v>
       </c>
-      <c r="H24" s="344">
+      <c r="H24" s="204">
         <v>2</v>
       </c>
-      <c r="I24" s="344">
+      <c r="I24" s="204">
         <v>1</v>
       </c>
-      <c r="J24" s="344" t="s">
+      <c r="J24" s="204" t="s">
         <v>252</v>
       </c>
-      <c r="K24" s="344">
+      <c r="K24" s="204">
         <v>1</v>
       </c>
-      <c r="L24" s="344">
+      <c r="L24" s="204">
         <v>3</v>
       </c>
-      <c r="M24" s="344">
+      <c r="M24" s="204">
         <v>2</v>
       </c>
     </row>
     <row r="25" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B25" s="337"/>
-      <c r="C25" s="337"/>
-      <c r="D25" s="335">
+      <c r="B25" s="199"/>
+      <c r="C25" s="199"/>
+      <c r="D25" s="197">
         <f>D13</f>
         <v>0</v>
       </c>
-      <c r="E25" s="338"/>
-      <c r="F25" s="338"/>
-      <c r="G25" s="338"/>
-      <c r="H25" s="338"/>
-      <c r="I25" s="338"/>
-      <c r="J25" s="339"/>
-      <c r="K25" s="338"/>
-      <c r="L25" s="338"/>
-      <c r="M25" s="338"/>
+      <c r="E25" s="200"/>
+      <c r="F25" s="200"/>
+      <c r="G25" s="200"/>
+      <c r="H25" s="200"/>
+      <c r="I25" s="200"/>
+      <c r="J25" s="201"/>
+      <c r="K25" s="200"/>
+      <c r="L25" s="200"/>
+      <c r="M25" s="200"/>
     </row>
     <row r="26" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B26" s="340" t="s">
+      <c r="B26" s="212" t="s">
         <v>42</v>
       </c>
-      <c r="C26" s="334"/>
-      <c r="D26" s="334"/>
-      <c r="E26" s="337">
+      <c r="C26" s="211"/>
+      <c r="D26" s="211"/>
+      <c r="E26" s="199">
         <f t="shared" ref="E26:M26" si="5">IFERROR(AVERAGE(E20:E24),2)</f>
         <v>3</v>
       </c>
-      <c r="F26" s="337">
+      <c r="F26" s="199">
         <f t="shared" si="5"/>
         <v>2.4</v>
       </c>
-      <c r="G26" s="337">
+      <c r="G26" s="199">
         <f t="shared" si="5"/>
         <v>2.6</v>
       </c>
-      <c r="H26" s="337">
+      <c r="H26" s="199">
         <f t="shared" si="5"/>
         <v>1.8</v>
       </c>
-      <c r="I26" s="337">
+      <c r="I26" s="199">
         <f t="shared" si="5"/>
         <v>1</v>
       </c>
-      <c r="J26" s="337">
+      <c r="J26" s="199">
         <f t="shared" si="5"/>
         <v>2</v>
       </c>
-      <c r="K26" s="337">
+      <c r="K26" s="199">
         <f t="shared" si="5"/>
         <v>1</v>
       </c>
-      <c r="L26" s="337">
+      <c r="L26" s="199">
         <f t="shared" si="5"/>
         <v>3</v>
       </c>
-      <c r="M26" s="337">
+      <c r="M26" s="199">
         <f t="shared" si="5"/>
         <v>2</v>
       </c>
     </row>
     <row r="27" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B27" s="341" t="s">
+      <c r="B27" s="213" t="s">
         <v>43</v>
       </c>
-      <c r="C27" s="334"/>
-      <c r="D27" s="334"/>
-      <c r="E27" s="342">
+      <c r="C27" s="211"/>
+      <c r="D27" s="211"/>
+      <c r="E27" s="202">
         <f t="shared" ref="E27:M27" si="6">E26</f>
         <v>3</v>
       </c>
-      <c r="F27" s="342">
+      <c r="F27" s="202">
         <f t="shared" si="6"/>
         <v>2.4</v>
       </c>
-      <c r="G27" s="342">
+      <c r="G27" s="202">
         <f t="shared" si="6"/>
         <v>2.6</v>
       </c>
-      <c r="H27" s="343">
+      <c r="H27" s="203">
         <f t="shared" si="6"/>
         <v>1.8</v>
       </c>
-      <c r="I27" s="343">
+      <c r="I27" s="203">
         <f t="shared" si="6"/>
         <v>1</v>
       </c>
-      <c r="J27" s="342">
+      <c r="J27" s="202">
         <f t="shared" si="6"/>
         <v>2</v>
       </c>
-      <c r="K27" s="342">
+      <c r="K27" s="202">
         <f t="shared" si="6"/>
         <v>1</v>
       </c>
-      <c r="L27" s="342">
+      <c r="L27" s="202">
         <f t="shared" si="6"/>
         <v>3</v>
       </c>
-      <c r="M27" s="342">
+      <c r="M27" s="202">
         <f t="shared" si="6"/>
         <v>2</v>
       </c>
@@ -4864,13 +4858,13 @@
       <c r="D30" s="25" t="s">
         <v>44</v>
       </c>
-      <c r="I30" s="208" t="s">
+      <c r="I30" s="207" t="s">
         <v>45</v>
       </c>
-      <c r="J30" s="206"/>
-      <c r="K30" s="206"/>
-      <c r="L30" s="206"/>
-      <c r="M30" s="206"/>
+      <c r="J30" s="208"/>
+      <c r="K30" s="208"/>
+      <c r="L30" s="208"/>
+      <c r="M30" s="208"/>
     </row>
     <row r="31" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="26"/>
@@ -4878,18 +4872,18 @@
       <c r="C31" s="209" t="s">
         <v>46</v>
       </c>
-      <c r="D31" s="210"/>
-      <c r="E31" s="210"/>
+      <c r="D31" s="206"/>
+      <c r="E31" s="206"/>
       <c r="F31" s="26"/>
       <c r="G31" s="26"/>
       <c r="H31" s="26"/>
       <c r="I31" s="209" t="s">
         <v>46</v>
       </c>
-      <c r="J31" s="210"/>
-      <c r="K31" s="210"/>
-      <c r="L31" s="210"/>
-      <c r="M31" s="210"/>
+      <c r="J31" s="206"/>
+      <c r="K31" s="206"/>
+      <c r="L31" s="206"/>
+      <c r="M31" s="206"/>
       <c r="N31" s="26"/>
       <c r="O31" s="26"/>
       <c r="P31" s="26"/>
@@ -4907,22 +4901,22 @@
     <row r="33" spans="2:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="34" spans="2:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="35" spans="2:5" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B35" s="203" t="s">
+      <c r="B35" s="214" t="s">
         <v>47</v>
       </c>
       <c r="C35" s="22"/>
-      <c r="D35" s="205" t="s">
+      <c r="D35" s="216" t="s">
         <v>48</v>
       </c>
-      <c r="E35" s="206"/>
+      <c r="E35" s="208"/>
     </row>
     <row r="36" spans="2:5" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B36" s="204"/>
+      <c r="B36" s="215"/>
       <c r="C36" s="24"/>
-      <c r="D36" s="207" t="s">
+      <c r="D36" s="217" t="s">
         <v>49</v>
       </c>
-      <c r="E36" s="206"/>
+      <c r="E36" s="208"/>
     </row>
     <row r="37" spans="2:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="38" spans="2:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -5892,11 +5886,9 @@
     <row r="1002" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="16">
-    <mergeCell ref="D3:E3"/>
-    <mergeCell ref="D4:E4"/>
-    <mergeCell ref="D5:E5"/>
-    <mergeCell ref="D6:E6"/>
-    <mergeCell ref="I30:M30"/>
+    <mergeCell ref="B35:B36"/>
+    <mergeCell ref="D35:E35"/>
+    <mergeCell ref="D36:E36"/>
     <mergeCell ref="C31:E31"/>
     <mergeCell ref="I31:M31"/>
     <mergeCell ref="B17:B19"/>
@@ -5905,9 +5897,11 @@
     <mergeCell ref="C17:D19"/>
     <mergeCell ref="B26:D26"/>
     <mergeCell ref="B27:D27"/>
-    <mergeCell ref="B35:B36"/>
-    <mergeCell ref="D35:E35"/>
-    <mergeCell ref="D36:E36"/>
+    <mergeCell ref="D3:E3"/>
+    <mergeCell ref="D4:E4"/>
+    <mergeCell ref="D5:E5"/>
+    <mergeCell ref="D6:E6"/>
+    <mergeCell ref="I30:M30"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup scale="69" orientation="landscape"/>
@@ -5916,7 +5910,7 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{12ADE8FF-0A50-48A3-9080-05C136E37F16}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <tabColor rgb="FFFFFF00"/>
   </sheetPr>
@@ -5927,243 +5921,243 @@
   </cols>
   <sheetData>
     <row r="5" spans="1:11" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B5" s="331" t="s">
+      <c r="B5" s="195" t="s">
         <v>250</v>
       </c>
-      <c r="C5" s="331" t="s">
+      <c r="C5" s="195" t="s">
         <v>24</v>
       </c>
-      <c r="D5" s="331" t="s">
+      <c r="D5" s="195" t="s">
         <v>25</v>
       </c>
-      <c r="E5" s="331" t="s">
+      <c r="E5" s="195" t="s">
         <v>26</v>
       </c>
-      <c r="F5" s="331" t="s">
+      <c r="F5" s="195" t="s">
         <v>27</v>
       </c>
-      <c r="G5" s="331" t="s">
+      <c r="G5" s="195" t="s">
         <v>28</v>
       </c>
-      <c r="H5" s="331" t="s">
+      <c r="H5" s="195" t="s">
         <v>29</v>
       </c>
-      <c r="I5" s="331" t="s">
+      <c r="I5" s="195" t="s">
         <v>30</v>
       </c>
-      <c r="J5" s="331" t="s">
+      <c r="J5" s="195" t="s">
         <v>31</v>
       </c>
-      <c r="K5" s="331" t="s">
+      <c r="K5" s="195" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="6" spans="1:11" ht="46.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B6" s="331" t="s">
+      <c r="B6" s="195" t="s">
         <v>251</v>
       </c>
-      <c r="C6" s="332">
+      <c r="C6" s="196">
         <v>3</v>
       </c>
-      <c r="D6" s="332">
+      <c r="D6" s="196">
         <v>2</v>
       </c>
-      <c r="E6" s="332">
+      <c r="E6" s="196">
         <v>2</v>
       </c>
-      <c r="F6" s="332">
+      <c r="F6" s="196">
         <v>1</v>
       </c>
-      <c r="G6" s="332" t="s">
+      <c r="G6" s="196" t="s">
         <v>252</v>
       </c>
-      <c r="H6" s="332" t="s">
+      <c r="H6" s="196" t="s">
         <v>252</v>
       </c>
-      <c r="I6" s="332" t="s">
+      <c r="I6" s="196" t="s">
         <v>252</v>
       </c>
-      <c r="J6" s="332">
+      <c r="J6" s="196">
         <v>3</v>
       </c>
-      <c r="K6" s="332">
+      <c r="K6" s="196">
         <v>2</v>
       </c>
     </row>
     <row r="7" spans="1:11" ht="46.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B7" s="331" t="s">
+      <c r="B7" s="195" t="s">
         <v>253</v>
       </c>
-      <c r="C7" s="332">
+      <c r="C7" s="196">
         <v>3</v>
       </c>
-      <c r="D7" s="332">
+      <c r="D7" s="196">
         <v>3</v>
       </c>
-      <c r="E7" s="332">
+      <c r="E7" s="196">
         <v>2</v>
       </c>
-      <c r="F7" s="332">
+      <c r="F7" s="196">
         <v>2</v>
       </c>
-      <c r="G7" s="332" t="s">
+      <c r="G7" s="196" t="s">
         <v>252</v>
       </c>
-      <c r="H7" s="332" t="s">
+      <c r="H7" s="196" t="s">
         <v>252</v>
       </c>
-      <c r="I7" s="332">
+      <c r="I7" s="196">
         <v>1</v>
       </c>
-      <c r="J7" s="332">
+      <c r="J7" s="196">
         <v>3</v>
       </c>
-      <c r="K7" s="332">
+      <c r="K7" s="196">
         <v>2</v>
       </c>
     </row>
     <row r="8" spans="1:11" ht="46.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B8" s="331" t="s">
+      <c r="B8" s="195" t="s">
         <v>254</v>
       </c>
-      <c r="C8" s="332">
+      <c r="C8" s="196">
         <v>3</v>
       </c>
-      <c r="D8" s="332">
+      <c r="D8" s="196">
         <v>2</v>
       </c>
-      <c r="E8" s="332">
+      <c r="E8" s="196">
         <v>3</v>
       </c>
-      <c r="F8" s="332">
+      <c r="F8" s="196">
         <v>2</v>
       </c>
-      <c r="G8" s="332" t="s">
+      <c r="G8" s="196" t="s">
         <v>252</v>
       </c>
-      <c r="H8" s="332" t="s">
+      <c r="H8" s="196" t="s">
         <v>252</v>
       </c>
-      <c r="I8" s="332" t="s">
+      <c r="I8" s="196" t="s">
         <v>252</v>
       </c>
-      <c r="J8" s="332">
+      <c r="J8" s="196">
         <v>3</v>
       </c>
-      <c r="K8" s="332">
+      <c r="K8" s="196">
         <v>2</v>
       </c>
     </row>
     <row r="9" spans="1:11" ht="46.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B9" s="331" t="s">
+      <c r="B9" s="195" t="s">
         <v>255</v>
       </c>
-      <c r="C9" s="332">
+      <c r="C9" s="196">
         <v>3</v>
       </c>
-      <c r="D9" s="332">
+      <c r="D9" s="196">
         <v>2</v>
       </c>
-      <c r="E9" s="332">
+      <c r="E9" s="196">
         <v>3</v>
       </c>
-      <c r="F9" s="332">
+      <c r="F9" s="196">
         <v>2</v>
       </c>
-      <c r="G9" s="332" t="s">
+      <c r="G9" s="196" t="s">
         <v>252</v>
       </c>
-      <c r="H9" s="332" t="s">
+      <c r="H9" s="196" t="s">
         <v>252</v>
       </c>
-      <c r="I9" s="332" t="s">
+      <c r="I9" s="196" t="s">
         <v>252</v>
       </c>
-      <c r="J9" s="332">
+      <c r="J9" s="196">
         <v>3</v>
       </c>
-      <c r="K9" s="332">
+      <c r="K9" s="196">
         <v>2</v>
       </c>
     </row>
     <row r="10" spans="1:11" ht="46.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B10" s="331" t="s">
+      <c r="B10" s="195" t="s">
         <v>256</v>
       </c>
-      <c r="C10" s="332">
+      <c r="C10" s="196">
         <v>3</v>
       </c>
-      <c r="D10" s="332">
+      <c r="D10" s="196">
         <v>3</v>
       </c>
-      <c r="E10" s="332">
+      <c r="E10" s="196">
         <v>3</v>
       </c>
-      <c r="F10" s="332">
+      <c r="F10" s="196">
         <v>2</v>
       </c>
-      <c r="G10" s="332">
+      <c r="G10" s="196">
         <v>1</v>
       </c>
-      <c r="H10" s="332" t="s">
+      <c r="H10" s="196" t="s">
         <v>252</v>
       </c>
-      <c r="I10" s="332">
+      <c r="I10" s="196">
         <v>1</v>
       </c>
-      <c r="J10" s="332">
+      <c r="J10" s="196">
         <v>3</v>
       </c>
-      <c r="K10" s="332">
+      <c r="K10" s="196">
         <v>2</v>
       </c>
     </row>
     <row r="13" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="14" spans="1:11" ht="23.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="329" t="s">
+      <c r="A14" s="193" t="s">
         <v>21</v>
       </c>
-      <c r="B14" s="329" t="s">
+      <c r="B14" s="193" t="s">
         <v>257</v>
       </c>
     </row>
     <row r="15" spans="1:11" ht="59.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="329" t="s">
+      <c r="A15" s="193" t="s">
         <v>9</v>
       </c>
-      <c r="B15" s="330" t="s">
+      <c r="B15" s="194" t="s">
         <v>258</v>
       </c>
     </row>
-    <row r="16" spans="1:11" ht="59.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="329" t="s">
+    <row r="16" spans="1:11" ht="45" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="193" t="s">
         <v>11</v>
       </c>
-      <c r="B16" s="330" t="s">
+      <c r="B16" s="194" t="s">
         <v>259</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="59.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="329" t="s">
+    <row r="17" spans="1:2" ht="45" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="193" t="s">
         <v>12</v>
       </c>
-      <c r="B17" s="330" t="s">
+      <c r="B17" s="194" t="s">
         <v>260</v>
       </c>
     </row>
     <row r="18" spans="1:2" ht="59.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="329" t="s">
+      <c r="A18" s="193" t="s">
         <v>14</v>
       </c>
-      <c r="B18" s="330" t="s">
+      <c r="B18" s="194" t="s">
         <v>261</v>
       </c>
     </row>
     <row r="19" spans="1:2" ht="59.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="329" t="s">
+      <c r="A19" s="193" t="s">
         <v>16</v>
       </c>
-      <c r="B19" s="330" t="s">
+      <c r="B19" s="194" t="s">
         <v>262</v>
       </c>
     </row>
@@ -6173,7 +6167,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <tabColor rgb="FFFFFF00"/>
   </sheetPr>
@@ -6195,38 +6189,38 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="21.75" x14ac:dyDescent="0.35">
-      <c r="A1" s="240" t="s">
+      <c r="A1" s="227" t="s">
         <v>50</v>
       </c>
-      <c r="B1" s="206"/>
-      <c r="C1" s="206"/>
-      <c r="D1" s="206"/>
-      <c r="E1" s="206"/>
-      <c r="F1" s="206"/>
-      <c r="G1" s="206"/>
-      <c r="H1" s="206"/>
-      <c r="I1" s="206"/>
-      <c r="J1" s="206"/>
-      <c r="K1" s="206"/>
+      <c r="B1" s="208"/>
+      <c r="C1" s="208"/>
+      <c r="D1" s="208"/>
+      <c r="E1" s="208"/>
+      <c r="F1" s="208"/>
+      <c r="G1" s="208"/>
+      <c r="H1" s="208"/>
+      <c r="I1" s="208"/>
+      <c r="J1" s="208"/>
+      <c r="K1" s="208"/>
       <c r="L1" s="27"/>
       <c r="M1" s="27"/>
       <c r="N1" s="27"/>
       <c r="O1" s="27"/>
     </row>
     <row r="2" spans="1:15" ht="21.75" x14ac:dyDescent="0.35">
-      <c r="A2" s="240" t="s">
+      <c r="A2" s="227" t="s">
         <v>51</v>
       </c>
-      <c r="B2" s="206"/>
-      <c r="C2" s="206"/>
-      <c r="D2" s="206"/>
-      <c r="E2" s="206"/>
-      <c r="F2" s="206"/>
-      <c r="G2" s="206"/>
-      <c r="H2" s="206"/>
-      <c r="I2" s="206"/>
-      <c r="J2" s="206"/>
-      <c r="K2" s="206"/>
+      <c r="B2" s="208"/>
+      <c r="C2" s="208"/>
+      <c r="D2" s="208"/>
+      <c r="E2" s="208"/>
+      <c r="F2" s="208"/>
+      <c r="G2" s="208"/>
+      <c r="H2" s="208"/>
+      <c r="I2" s="208"/>
+      <c r="J2" s="208"/>
+      <c r="K2" s="208"/>
       <c r="L2" s="27"/>
       <c r="M2" s="27"/>
       <c r="N2" s="27"/>
@@ -6237,11 +6231,11 @@
       <c r="B3" s="28" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="241" t="str">
+      <c r="C3" s="228" t="str">
         <f>'PO Set Target attain level'!D3</f>
         <v>Data Structures Using _C</v>
       </c>
-      <c r="D3" s="242"/>
+      <c r="D3" s="229"/>
       <c r="E3" s="27"/>
       <c r="F3" s="27"/>
       <c r="G3" s="27"/>
@@ -6259,11 +6253,11 @@
       <c r="B4" s="28" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="241">
+      <c r="C4" s="228">
         <f>'PO Set Target attain level'!D4</f>
         <v>22317</v>
       </c>
-      <c r="D4" s="242"/>
+      <c r="D4" s="229"/>
       <c r="E4" s="27"/>
       <c r="F4" s="27"/>
       <c r="G4" s="27"/>
@@ -6281,11 +6275,11 @@
       <c r="B5" s="28" t="s">
         <v>52</v>
       </c>
-      <c r="C5" s="241" t="str">
+      <c r="C5" s="228" t="str">
         <f>'PO Set Target attain level'!D5</f>
         <v>3rd SEM(CO3I SCHEME)</v>
       </c>
-      <c r="D5" s="242"/>
+      <c r="D5" s="229"/>
       <c r="E5" s="27"/>
       <c r="F5" s="27"/>
       <c r="G5" s="27"/>
@@ -6303,11 +6297,11 @@
       <c r="B6" s="28" t="s">
         <v>53</v>
       </c>
-      <c r="C6" s="241" t="str">
+      <c r="C6" s="228" t="str">
         <f>'PO Set Target attain level'!D6</f>
         <v>2023-24</v>
       </c>
-      <c r="D6" s="242"/>
+      <c r="D6" s="229"/>
       <c r="E6" s="27"/>
       <c r="F6" s="27"/>
       <c r="G6" s="27"/>
@@ -6338,31 +6332,31 @@
       <c r="O7" s="27"/>
     </row>
     <row r="8" spans="1:15" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="243" t="s">
+      <c r="A8" s="230" t="s">
         <v>20</v>
       </c>
-      <c r="B8" s="220" t="s">
+      <c r="B8" s="260" t="s">
         <v>54</v>
       </c>
-      <c r="C8" s="221" t="s">
+      <c r="C8" s="261" t="s">
         <v>55</v>
       </c>
-      <c r="D8" s="236" t="s">
+      <c r="D8" s="264" t="s">
         <v>56</v>
       </c>
-      <c r="E8" s="237" t="s">
+      <c r="E8" s="265" t="s">
         <v>57</v>
       </c>
-      <c r="F8" s="216" t="s">
+      <c r="F8" s="258" t="s">
         <v>58</v>
       </c>
-      <c r="G8" s="219" t="s">
+      <c r="G8" s="259" t="s">
         <v>59</v>
       </c>
-      <c r="H8" s="238" t="s">
+      <c r="H8" s="223" t="s">
         <v>60</v>
       </c>
-      <c r="I8" s="239" t="s">
+      <c r="I8" s="226" t="s">
         <v>61</v>
       </c>
       <c r="J8" s="29" t="s">
@@ -6377,62 +6371,62 @@
       <c r="O8" s="27"/>
     </row>
     <row r="9" spans="1:15" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="217"/>
-      <c r="B9" s="217"/>
-      <c r="C9" s="217"/>
-      <c r="D9" s="217"/>
-      <c r="E9" s="217"/>
-      <c r="F9" s="217"/>
-      <c r="G9" s="217"/>
-      <c r="H9" s="217"/>
-      <c r="I9" s="217"/>
-      <c r="J9" s="244" t="s">
+      <c r="A9" s="224"/>
+      <c r="B9" s="224"/>
+      <c r="C9" s="224"/>
+      <c r="D9" s="224"/>
+      <c r="E9" s="224"/>
+      <c r="F9" s="224"/>
+      <c r="G9" s="224"/>
+      <c r="H9" s="224"/>
+      <c r="I9" s="224"/>
+      <c r="J9" s="231" t="s">
         <v>64</v>
       </c>
-      <c r="K9" s="245"/>
+      <c r="K9" s="232"/>
       <c r="L9" s="27"/>
       <c r="M9" s="27"/>
       <c r="N9" s="27"/>
       <c r="O9" s="27"/>
     </row>
     <row r="10" spans="1:15" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="217"/>
-      <c r="B10" s="217"/>
-      <c r="C10" s="217"/>
-      <c r="D10" s="217"/>
-      <c r="E10" s="217"/>
-      <c r="F10" s="217"/>
-      <c r="G10" s="217"/>
-      <c r="H10" s="217"/>
-      <c r="I10" s="217"/>
-      <c r="J10" s="246"/>
-      <c r="K10" s="204"/>
+      <c r="A10" s="224"/>
+      <c r="B10" s="224"/>
+      <c r="C10" s="224"/>
+      <c r="D10" s="224"/>
+      <c r="E10" s="224"/>
+      <c r="F10" s="224"/>
+      <c r="G10" s="224"/>
+      <c r="H10" s="224"/>
+      <c r="I10" s="224"/>
+      <c r="J10" s="233"/>
+      <c r="K10" s="215"/>
       <c r="L10" s="27"/>
       <c r="M10" s="27"/>
       <c r="N10" s="27"/>
       <c r="O10" s="27"/>
     </row>
     <row r="11" spans="1:15" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="217"/>
-      <c r="B11" s="217"/>
-      <c r="C11" s="217"/>
-      <c r="D11" s="218"/>
-      <c r="E11" s="218"/>
-      <c r="F11" s="218"/>
-      <c r="G11" s="218"/>
-      <c r="H11" s="218"/>
-      <c r="I11" s="218"/>
-      <c r="J11" s="247"/>
-      <c r="K11" s="248"/>
+      <c r="A11" s="224"/>
+      <c r="B11" s="224"/>
+      <c r="C11" s="224"/>
+      <c r="D11" s="225"/>
+      <c r="E11" s="225"/>
+      <c r="F11" s="225"/>
+      <c r="G11" s="225"/>
+      <c r="H11" s="225"/>
+      <c r="I11" s="225"/>
+      <c r="J11" s="234"/>
+      <c r="K11" s="235"/>
       <c r="L11" s="27"/>
       <c r="M11" s="27"/>
       <c r="N11" s="27"/>
       <c r="O11" s="27"/>
     </row>
     <row r="12" spans="1:15" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="218"/>
-      <c r="B12" s="218"/>
-      <c r="C12" s="218"/>
+      <c r="A12" s="225"/>
+      <c r="B12" s="225"/>
+      <c r="C12" s="225"/>
       <c r="D12" s="30"/>
       <c r="E12" s="31"/>
       <c r="F12" s="31"/>
@@ -8859,93 +8853,93 @@
       <c r="O94" s="27"/>
     </row>
     <row r="95" spans="1:15" ht="60.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A95" s="222" t="s">
+      <c r="A95" s="262" t="s">
         <v>133</v>
       </c>
-      <c r="B95" s="206"/>
+      <c r="B95" s="208"/>
       <c r="C95" s="50">
         <v>0.4</v>
       </c>
-      <c r="D95" s="223">
+      <c r="D95" s="218">
         <f t="shared" ref="D95:I95" si="8">$C$95*D12</f>
         <v>0</v>
       </c>
-      <c r="E95" s="223">
+      <c r="E95" s="218">
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
-      <c r="F95" s="223">
+      <c r="F95" s="218">
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
-      <c r="G95" s="223">
+      <c r="G95" s="218">
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
-      <c r="H95" s="223">
+      <c r="H95" s="218">
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
-      <c r="I95" s="223">
+      <c r="I95" s="218">
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
-      <c r="J95" s="249"/>
-      <c r="K95" s="249"/>
+      <c r="J95" s="220"/>
+      <c r="K95" s="220"/>
       <c r="L95" s="27"/>
       <c r="M95" s="27"/>
       <c r="N95" s="27"/>
       <c r="O95" s="27"/>
     </row>
     <row r="96" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A96" s="224" t="s">
+      <c r="A96" s="263" t="s">
         <v>134</v>
       </c>
-      <c r="B96" s="206"/>
-      <c r="C96" s="196"/>
-      <c r="D96" s="213"/>
-      <c r="E96" s="213"/>
-      <c r="F96" s="213"/>
-      <c r="G96" s="213"/>
-      <c r="H96" s="213"/>
-      <c r="I96" s="213"/>
-      <c r="J96" s="213"/>
-      <c r="K96" s="213"/>
+      <c r="B96" s="208"/>
+      <c r="C96" s="251"/>
+      <c r="D96" s="219"/>
+      <c r="E96" s="219"/>
+      <c r="F96" s="219"/>
+      <c r="G96" s="219"/>
+      <c r="H96" s="219"/>
+      <c r="I96" s="219"/>
+      <c r="J96" s="219"/>
+      <c r="K96" s="219"/>
       <c r="L96" s="27"/>
       <c r="M96" s="27"/>
       <c r="N96" s="27"/>
       <c r="O96" s="27"/>
     </row>
     <row r="97" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A97" s="206"/>
-      <c r="B97" s="206"/>
-      <c r="C97" s="196"/>
-      <c r="D97" s="251">
+      <c r="A97" s="208"/>
+      <c r="B97" s="208"/>
+      <c r="C97" s="251"/>
+      <c r="D97" s="222">
         <f t="shared" ref="D97:I97" si="9">COUNTIF(D13:D94,"&gt;=" &amp;D95)</f>
         <v>0</v>
       </c>
-      <c r="E97" s="251">
+      <c r="E97" s="222">
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
-      <c r="F97" s="251">
+      <c r="F97" s="222">
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
-      <c r="G97" s="251">
+      <c r="G97" s="222">
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
-      <c r="H97" s="251">
+      <c r="H97" s="222">
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
-      <c r="I97" s="251">
+      <c r="I97" s="222">
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
-      <c r="J97" s="250"/>
-      <c r="K97" s="250"/>
+      <c r="J97" s="221"/>
+      <c r="K97" s="221"/>
       <c r="L97" s="27"/>
       <c r="M97" s="27"/>
       <c r="N97" s="27"/>
@@ -8955,14 +8949,14 @@
       <c r="A98" s="27"/>
       <c r="B98" s="27"/>
       <c r="C98" s="27"/>
-      <c r="D98" s="213"/>
-      <c r="E98" s="213"/>
-      <c r="F98" s="213"/>
-      <c r="G98" s="213"/>
-      <c r="H98" s="213"/>
-      <c r="I98" s="213"/>
-      <c r="J98" s="213"/>
-      <c r="K98" s="213"/>
+      <c r="D98" s="219"/>
+      <c r="E98" s="219"/>
+      <c r="F98" s="219"/>
+      <c r="G98" s="219"/>
+      <c r="H98" s="219"/>
+      <c r="I98" s="219"/>
+      <c r="J98" s="219"/>
+      <c r="K98" s="219"/>
       <c r="L98" s="27"/>
       <c r="M98" s="27"/>
       <c r="N98" s="27"/>
@@ -9021,21 +9015,21 @@
     </row>
     <row r="102" spans="1:15" ht="43.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A102" s="27"/>
-      <c r="B102" s="229" t="s">
+      <c r="B102" s="241" t="s">
         <v>135</v>
       </c>
-      <c r="C102" s="200"/>
-      <c r="D102" s="200"/>
-      <c r="E102" s="201"/>
-      <c r="F102" s="230" t="s">
+      <c r="C102" s="237"/>
+      <c r="D102" s="237"/>
+      <c r="E102" s="242"/>
+      <c r="F102" s="243" t="s">
         <v>136</v>
       </c>
-      <c r="G102" s="201"/>
+      <c r="G102" s="242"/>
       <c r="H102" s="51"/>
-      <c r="I102" s="231" t="s">
+      <c r="I102" s="244" t="s">
         <v>137</v>
       </c>
-      <c r="J102" s="201"/>
+      <c r="J102" s="242"/>
       <c r="K102" s="27"/>
       <c r="L102" s="27"/>
       <c r="M102" s="27"/>
@@ -9044,28 +9038,28 @@
     </row>
     <row r="103" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A103" s="27"/>
-      <c r="B103" s="232" t="s">
+      <c r="B103" s="245" t="s">
         <v>138</v>
       </c>
-      <c r="C103" s="225" t="s">
+      <c r="C103" s="236" t="s">
         <v>139</v>
       </c>
-      <c r="D103" s="200"/>
+      <c r="D103" s="237"/>
       <c r="E103" s="52">
         <v>50</v>
       </c>
-      <c r="F103" s="235">
+      <c r="F103" s="248">
         <v>62</v>
       </c>
-      <c r="G103" s="194"/>
+      <c r="G103" s="249"/>
       <c r="H103" s="53">
         <f>E103*F103/100</f>
         <v>31</v>
       </c>
-      <c r="I103" s="252">
+      <c r="I103" s="254">
         <v>1</v>
       </c>
-      <c r="J103" s="253"/>
+      <c r="J103" s="255"/>
       <c r="K103" s="27"/>
       <c r="L103" s="27"/>
       <c r="M103" s="27"/>
@@ -9074,24 +9068,24 @@
     </row>
     <row r="104" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A104" s="27"/>
-      <c r="B104" s="233"/>
-      <c r="C104" s="225" t="s">
+      <c r="B104" s="246"/>
+      <c r="C104" s="236" t="s">
         <v>139</v>
       </c>
-      <c r="D104" s="200"/>
+      <c r="D104" s="237"/>
       <c r="E104" s="52">
         <v>60</v>
       </c>
-      <c r="F104" s="195"/>
-      <c r="G104" s="196"/>
+      <c r="F104" s="250"/>
+      <c r="G104" s="251"/>
       <c r="H104" s="54">
         <f>E104*F103/100</f>
         <v>37.200000000000003</v>
       </c>
-      <c r="I104" s="254">
+      <c r="I104" s="256">
         <v>2</v>
       </c>
-      <c r="J104" s="255"/>
+      <c r="J104" s="257"/>
       <c r="K104" s="27"/>
       <c r="L104" s="27"/>
       <c r="M104" s="27"/>
@@ -9100,24 +9094,24 @@
     </row>
     <row r="105" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A105" s="27"/>
-      <c r="B105" s="234"/>
-      <c r="C105" s="225" t="s">
+      <c r="B105" s="247"/>
+      <c r="C105" s="236" t="s">
         <v>139</v>
       </c>
-      <c r="D105" s="200"/>
+      <c r="D105" s="237"/>
       <c r="E105" s="55">
         <v>70</v>
       </c>
-      <c r="F105" s="197"/>
-      <c r="G105" s="198"/>
+      <c r="F105" s="252"/>
+      <c r="G105" s="253"/>
       <c r="H105" s="56">
         <f>E105*F103/100</f>
         <v>43.4</v>
       </c>
-      <c r="I105" s="226">
+      <c r="I105" s="238">
         <v>3</v>
       </c>
-      <c r="J105" s="227"/>
+      <c r="J105" s="239"/>
       <c r="K105" s="27"/>
       <c r="L105" s="27"/>
       <c r="M105" s="27"/>
@@ -9132,9 +9126,9 @@
       <c r="E106" s="57"/>
       <c r="F106" s="57"/>
       <c r="G106" s="57"/>
-      <c r="H106" s="228"/>
-      <c r="I106" s="210"/>
-      <c r="J106" s="210"/>
+      <c r="H106" s="240"/>
+      <c r="I106" s="206"/>
+      <c r="J106" s="206"/>
       <c r="K106" s="27"/>
       <c r="L106" s="27"/>
       <c r="M106" s="27"/>
@@ -9149,9 +9143,9 @@
       <c r="E107" s="57"/>
       <c r="F107" s="57"/>
       <c r="G107" s="57"/>
-      <c r="H107" s="228"/>
-      <c r="I107" s="210"/>
-      <c r="J107" s="210"/>
+      <c r="H107" s="240"/>
+      <c r="I107" s="206"/>
+      <c r="J107" s="206"/>
       <c r="K107" s="27"/>
       <c r="L107" s="27"/>
       <c r="M107" s="27"/>
@@ -13496,24 +13490,16 @@
     <row r="999" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="47">
-    <mergeCell ref="H95:H96"/>
-    <mergeCell ref="I95:I96"/>
-    <mergeCell ref="J95:J96"/>
-    <mergeCell ref="K95:K96"/>
-    <mergeCell ref="J97:J98"/>
-    <mergeCell ref="K97:K98"/>
-    <mergeCell ref="H97:H98"/>
-    <mergeCell ref="I97:I98"/>
-    <mergeCell ref="H8:H11"/>
-    <mergeCell ref="I8:I11"/>
-    <mergeCell ref="A1:K1"/>
-    <mergeCell ref="A2:K2"/>
-    <mergeCell ref="C3:D3"/>
-    <mergeCell ref="C4:D4"/>
-    <mergeCell ref="C5:D5"/>
-    <mergeCell ref="C6:D6"/>
-    <mergeCell ref="A8:A12"/>
-    <mergeCell ref="J9:K11"/>
+    <mergeCell ref="A95:B95"/>
+    <mergeCell ref="E95:E96"/>
+    <mergeCell ref="F95:F96"/>
+    <mergeCell ref="G95:G96"/>
+    <mergeCell ref="A96:C97"/>
+    <mergeCell ref="D95:D96"/>
+    <mergeCell ref="D97:D98"/>
+    <mergeCell ref="E97:E98"/>
+    <mergeCell ref="F97:F98"/>
+    <mergeCell ref="G97:G98"/>
     <mergeCell ref="C105:D105"/>
     <mergeCell ref="I105:J105"/>
     <mergeCell ref="H106:J106"/>
@@ -13527,22 +13513,30 @@
     <mergeCell ref="C104:D104"/>
     <mergeCell ref="I103:J103"/>
     <mergeCell ref="I104:J104"/>
+    <mergeCell ref="H8:H11"/>
+    <mergeCell ref="I8:I11"/>
+    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="C3:D3"/>
+    <mergeCell ref="C4:D4"/>
+    <mergeCell ref="C5:D5"/>
+    <mergeCell ref="C6:D6"/>
+    <mergeCell ref="A8:A12"/>
+    <mergeCell ref="J9:K11"/>
     <mergeCell ref="F8:F11"/>
     <mergeCell ref="G8:G11"/>
     <mergeCell ref="B8:B12"/>
     <mergeCell ref="C8:C12"/>
-    <mergeCell ref="A95:B95"/>
-    <mergeCell ref="E95:E96"/>
-    <mergeCell ref="F95:F96"/>
-    <mergeCell ref="G95:G96"/>
-    <mergeCell ref="A96:C97"/>
     <mergeCell ref="D8:D11"/>
     <mergeCell ref="E8:E11"/>
-    <mergeCell ref="D95:D96"/>
-    <mergeCell ref="D97:D98"/>
-    <mergeCell ref="E97:E98"/>
-    <mergeCell ref="F97:F98"/>
-    <mergeCell ref="G97:G98"/>
+    <mergeCell ref="H95:H96"/>
+    <mergeCell ref="I95:I96"/>
+    <mergeCell ref="J95:J96"/>
+    <mergeCell ref="K95:K96"/>
+    <mergeCell ref="J97:J98"/>
+    <mergeCell ref="K97:K98"/>
+    <mergeCell ref="H97:H98"/>
+    <mergeCell ref="I97:I98"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>
@@ -13551,7 +13545,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <tabColor rgb="FFFFFF00"/>
   </sheetPr>
@@ -13568,13 +13562,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:22" ht="20.25" x14ac:dyDescent="0.25">
-      <c r="B1" s="256" t="s">
+      <c r="B1" s="279" t="s">
         <v>145</v>
       </c>
-      <c r="C1" s="206"/>
-      <c r="D1" s="206"/>
-      <c r="E1" s="206"/>
-      <c r="F1" s="206"/>
+      <c r="C1" s="208"/>
+      <c r="D1" s="208"/>
+      <c r="E1" s="208"/>
+      <c r="F1" s="208"/>
       <c r="G1" s="27"/>
       <c r="H1" s="27"/>
       <c r="I1" s="27"/>
@@ -13643,11 +13637,11 @@
       <c r="C4" s="28" t="s">
         <v>1</v>
       </c>
-      <c r="D4" s="257" t="str">
+      <c r="D4" s="280" t="str">
         <f>'CO_Attainment for Unit Tests'!C3</f>
         <v>Data Structures Using _C</v>
       </c>
-      <c r="E4" s="210"/>
+      <c r="E4" s="206"/>
       <c r="F4" s="27"/>
       <c r="G4" s="27"/>
       <c r="H4" s="27"/>
@@ -13671,11 +13665,11 @@
       <c r="C5" s="28" t="s">
         <v>3</v>
       </c>
-      <c r="D5" s="257">
+      <c r="D5" s="280">
         <f>'CO_Attainment for Unit Tests'!C4</f>
         <v>22317</v>
       </c>
-      <c r="E5" s="210"/>
+      <c r="E5" s="206"/>
       <c r="F5" s="27"/>
       <c r="G5" s="27"/>
       <c r="H5" s="27"/>
@@ -13699,11 +13693,11 @@
       <c r="C6" s="28" t="s">
         <v>52</v>
       </c>
-      <c r="D6" s="257" t="str">
+      <c r="D6" s="280" t="str">
         <f>'CO_Attainment for Unit Tests'!C5</f>
         <v>3rd SEM(CO3I SCHEME)</v>
       </c>
-      <c r="E6" s="210"/>
+      <c r="E6" s="206"/>
       <c r="F6" s="27"/>
       <c r="G6" s="27"/>
       <c r="H6" s="27"/>
@@ -13727,11 +13721,11 @@
       <c r="C7" s="28" t="s">
         <v>6</v>
       </c>
-      <c r="D7" s="257" t="str">
+      <c r="D7" s="280" t="str">
         <f>'CO_Attainment for Unit Tests'!C6</f>
         <v>2023-24</v>
       </c>
-      <c r="E7" s="210"/>
+      <c r="E7" s="206"/>
       <c r="F7" s="27"/>
       <c r="G7" s="27"/>
       <c r="H7" s="27"/>
@@ -13754,43 +13748,43 @@
       <c r="E8" s="15"/>
     </row>
     <row r="9" spans="2:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B9" s="258" t="s">
+      <c r="B9" s="274" t="s">
         <v>20</v>
       </c>
-      <c r="C9" s="259" t="s">
+      <c r="C9" s="268" t="s">
         <v>54</v>
       </c>
-      <c r="D9" s="221" t="s">
+      <c r="D9" s="261" t="s">
         <v>55</v>
       </c>
-      <c r="E9" s="259" t="s">
+      <c r="E9" s="268" t="s">
         <v>147</v>
       </c>
       <c r="J9" s="64"/>
     </row>
     <row r="10" spans="2:22" x14ac:dyDescent="0.25">
-      <c r="B10" s="217"/>
-      <c r="C10" s="217"/>
-      <c r="D10" s="217"/>
-      <c r="E10" s="217"/>
+      <c r="B10" s="224"/>
+      <c r="C10" s="224"/>
+      <c r="D10" s="224"/>
+      <c r="E10" s="224"/>
       <c r="J10" s="65"/>
     </row>
     <row r="11" spans="2:22" x14ac:dyDescent="0.25">
-      <c r="B11" s="217"/>
-      <c r="C11" s="217"/>
-      <c r="D11" s="217"/>
-      <c r="E11" s="217"/>
+      <c r="B11" s="224"/>
+      <c r="C11" s="224"/>
+      <c r="D11" s="224"/>
+      <c r="E11" s="224"/>
     </row>
     <row r="12" spans="2:22" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B12" s="217"/>
-      <c r="C12" s="217"/>
-      <c r="D12" s="217"/>
-      <c r="E12" s="218"/>
+      <c r="B12" s="224"/>
+      <c r="C12" s="224"/>
+      <c r="D12" s="224"/>
+      <c r="E12" s="225"/>
     </row>
     <row r="13" spans="2:22" x14ac:dyDescent="0.25">
-      <c r="B13" s="218"/>
-      <c r="C13" s="218"/>
-      <c r="D13" s="218"/>
+      <c r="B13" s="225"/>
+      <c r="C13" s="225"/>
+      <c r="D13" s="225"/>
       <c r="E13" s="32">
         <v>70</v>
       </c>
@@ -15143,7 +15137,7 @@
       <c r="D97" s="69" t="s">
         <v>148</v>
       </c>
-      <c r="E97" s="266">
+      <c r="E97" s="269">
         <f>D98*E13/100</f>
         <v>32.878999999999998</v>
       </c>
@@ -15152,7 +15146,7 @@
       <c r="D98" s="70">
         <v>46.97</v>
       </c>
-      <c r="E98" s="213"/>
+      <c r="E98" s="219"/>
     </row>
     <row r="99" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D99" s="71" t="s">
@@ -15178,12 +15172,12 @@
       <c r="E102" s="15"/>
     </row>
     <row r="103" spans="1:9" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A103" s="229" t="s">
+      <c r="A103" s="241" t="s">
         <v>135</v>
       </c>
-      <c r="B103" s="200"/>
-      <c r="C103" s="200"/>
-      <c r="D103" s="201"/>
+      <c r="B103" s="237"/>
+      <c r="C103" s="237"/>
+      <c r="D103" s="242"/>
       <c r="E103" s="75" t="s">
         <v>136</v>
       </c>
@@ -15195,17 +15189,17 @@
       <c r="I103" s="77"/>
     </row>
     <row r="104" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A104" s="232" t="s">
+      <c r="A104" s="245" t="s">
         <v>138</v>
       </c>
       <c r="B104" s="78">
         <v>0.5</v>
       </c>
-      <c r="C104" s="267" t="s">
+      <c r="C104" s="270" t="s">
         <v>150</v>
       </c>
-      <c r="D104" s="268"/>
-      <c r="E104" s="269">
+      <c r="D104" s="271"/>
+      <c r="E104" s="272">
         <f>COUNTA(D14:D96)-COUNTIFS(D14:D96,0)</f>
         <v>62</v>
       </c>
@@ -15220,15 +15214,15 @@
       <c r="I104" s="77"/>
     </row>
     <row r="105" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A105" s="233"/>
+      <c r="A105" s="246"/>
       <c r="B105" s="81">
         <v>0.6</v>
       </c>
-      <c r="C105" s="260" t="s">
+      <c r="C105" s="275" t="s">
         <v>150</v>
       </c>
-      <c r="D105" s="255"/>
-      <c r="E105" s="212"/>
+      <c r="D105" s="257"/>
+      <c r="E105" s="273"/>
       <c r="F105" s="82">
         <f t="shared" si="0"/>
         <v>37.199999999999996</v>
@@ -15240,15 +15234,15 @@
       <c r="I105" s="77"/>
     </row>
     <row r="106" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A106" s="234"/>
+      <c r="A106" s="247"/>
       <c r="B106" s="84">
         <v>0.7</v>
       </c>
-      <c r="C106" s="261" t="s">
+      <c r="C106" s="276" t="s">
         <v>151</v>
       </c>
-      <c r="D106" s="227"/>
-      <c r="E106" s="213"/>
+      <c r="D106" s="239"/>
+      <c r="E106" s="219"/>
       <c r="F106" s="85">
         <f t="shared" si="0"/>
         <v>43.4</v>
@@ -15282,10 +15276,10 @@
       <c r="I108" s="77"/>
     </row>
     <row r="109" spans="1:9" ht="71.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A109" s="262" t="s">
+      <c r="A109" s="277" t="s">
         <v>152</v>
       </c>
-      <c r="B109" s="263"/>
+      <c r="B109" s="278"/>
       <c r="C109" s="59" t="s">
         <v>9</v>
       </c>
@@ -15307,10 +15301,10 @@
       <c r="I109" s="77"/>
     </row>
     <row r="110" spans="1:9" ht="39" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A110" s="264" t="s">
+      <c r="A110" s="266" t="s">
         <v>153</v>
       </c>
-      <c r="B110" s="265"/>
+      <c r="B110" s="267"/>
       <c r="C110" s="62">
         <f>IF(E99&gt;=$F106,3,IF(E99&gt;=$F105,2,IF(E99&gt;=$F104,1,0)))</f>
         <v>3</v>
@@ -16649,6 +16643,11 @@
     <row r="1000" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="18">
+    <mergeCell ref="B1:F1"/>
+    <mergeCell ref="D4:E4"/>
+    <mergeCell ref="D5:E5"/>
+    <mergeCell ref="D6:E6"/>
+    <mergeCell ref="D7:E7"/>
     <mergeCell ref="A110:B110"/>
     <mergeCell ref="D9:D13"/>
     <mergeCell ref="E9:E12"/>
@@ -16662,11 +16661,6 @@
     <mergeCell ref="C105:D105"/>
     <mergeCell ref="C106:D106"/>
     <mergeCell ref="A109:B109"/>
-    <mergeCell ref="B1:F1"/>
-    <mergeCell ref="D4:E4"/>
-    <mergeCell ref="D5:E5"/>
-    <mergeCell ref="D6:E6"/>
-    <mergeCell ref="D7:E7"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup orientation="portrait"/>
@@ -16675,7 +16669,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <tabColor rgb="FFFFFF00"/>
   </sheetPr>
@@ -16723,11 +16717,11 @@
       <c r="C4" s="28" t="s">
         <v>1</v>
       </c>
-      <c r="D4" s="241" t="str">
+      <c r="D4" s="228" t="str">
         <f>'CO_Attainment for Unit Tests'!C3</f>
         <v>Data Structures Using _C</v>
       </c>
-      <c r="E4" s="242"/>
+      <c r="E4" s="229"/>
       <c r="F4" s="27"/>
       <c r="G4" s="27"/>
       <c r="H4" s="27"/>
@@ -16737,11 +16731,11 @@
       <c r="C5" s="28" t="s">
         <v>3</v>
       </c>
-      <c r="D5" s="241">
+      <c r="D5" s="228">
         <f>'CO_Attainment for Unit Tests'!C4</f>
         <v>22317</v>
       </c>
-      <c r="E5" s="242"/>
+      <c r="E5" s="229"/>
       <c r="F5" s="27"/>
       <c r="G5" s="27"/>
       <c r="H5" s="27"/>
@@ -16751,11 +16745,11 @@
       <c r="C6" s="28" t="s">
         <v>52</v>
       </c>
-      <c r="D6" s="241" t="str">
+      <c r="D6" s="228" t="str">
         <f>'CO_Attainment for Unit Tests'!C5</f>
         <v>3rd SEM(CO3I SCHEME)</v>
       </c>
-      <c r="E6" s="242"/>
+      <c r="E6" s="229"/>
       <c r="F6" s="27"/>
       <c r="G6" s="27"/>
       <c r="H6" s="27"/>
@@ -16765,63 +16759,63 @@
       <c r="C7" s="28" t="s">
         <v>157</v>
       </c>
-      <c r="D7" s="241" t="str">
+      <c r="D7" s="228" t="str">
         <f>'CO_Attainment for Unit Tests'!C6</f>
         <v>2023-24</v>
       </c>
-      <c r="E7" s="242"/>
+      <c r="E7" s="229"/>
       <c r="F7" s="27"/>
       <c r="G7" s="27"/>
       <c r="H7" s="27"/>
     </row>
     <row r="9" spans="2:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B9" s="258" t="s">
+      <c r="B9" s="274" t="s">
         <v>20</v>
       </c>
-      <c r="C9" s="259" t="s">
+      <c r="C9" s="268" t="s">
         <v>54</v>
       </c>
-      <c r="D9" s="270" t="s">
+      <c r="D9" s="289" t="s">
         <v>55</v>
       </c>
-      <c r="E9" s="276" t="s">
+      <c r="E9" s="282" t="s">
         <v>158</v>
       </c>
-      <c r="F9" s="277" t="s">
+      <c r="F9" s="283" t="s">
         <v>159</v>
       </c>
-      <c r="G9" s="277" t="s">
+      <c r="G9" s="283" t="s">
         <v>160</v>
       </c>
     </row>
     <row r="10" spans="2:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B10" s="217"/>
-      <c r="C10" s="217"/>
-      <c r="D10" s="217"/>
-      <c r="E10" s="217"/>
-      <c r="F10" s="217"/>
-      <c r="G10" s="217"/>
+      <c r="B10" s="224"/>
+      <c r="C10" s="224"/>
+      <c r="D10" s="224"/>
+      <c r="E10" s="224"/>
+      <c r="F10" s="224"/>
+      <c r="G10" s="224"/>
     </row>
     <row r="11" spans="2:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B11" s="217"/>
-      <c r="C11" s="217"/>
-      <c r="D11" s="217"/>
-      <c r="E11" s="217"/>
-      <c r="F11" s="217"/>
-      <c r="G11" s="217"/>
+      <c r="B11" s="224"/>
+      <c r="C11" s="224"/>
+      <c r="D11" s="224"/>
+      <c r="E11" s="224"/>
+      <c r="F11" s="224"/>
+      <c r="G11" s="224"/>
     </row>
     <row r="12" spans="2:8" ht="54.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B12" s="217"/>
-      <c r="C12" s="217"/>
-      <c r="D12" s="217"/>
-      <c r="E12" s="218"/>
-      <c r="F12" s="218"/>
-      <c r="G12" s="218"/>
+      <c r="B12" s="224"/>
+      <c r="C12" s="224"/>
+      <c r="D12" s="224"/>
+      <c r="E12" s="225"/>
+      <c r="F12" s="225"/>
+      <c r="G12" s="225"/>
     </row>
     <row r="13" spans="2:8" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B13" s="218"/>
-      <c r="C13" s="218"/>
-      <c r="D13" s="218"/>
+      <c r="B13" s="225"/>
+      <c r="C13" s="225"/>
+      <c r="D13" s="225"/>
       <c r="E13" s="32">
         <v>10</v>
       </c>
@@ -18276,15 +18270,15 @@
       <c r="D97" s="90" t="s">
         <v>161</v>
       </c>
-      <c r="E97" s="271">
+      <c r="E97" s="284">
         <f>ROUNDUP(D98*E13/100,1)</f>
         <v>6</v>
       </c>
-      <c r="F97" s="271">
+      <c r="F97" s="284">
         <f>ROUNDUP(D98*F13/100,1)</f>
         <v>15</v>
       </c>
-      <c r="G97" s="271">
+      <c r="G97" s="284">
         <f>ROUNDUP(D98*G13/100,1)</f>
         <v>15</v>
       </c>
@@ -18293,9 +18287,9 @@
       <c r="D98" s="91">
         <v>60</v>
       </c>
-      <c r="E98" s="213"/>
-      <c r="F98" s="213"/>
-      <c r="G98" s="213"/>
+      <c r="E98" s="219"/>
+      <c r="F98" s="219"/>
+      <c r="G98" s="219"/>
     </row>
     <row r="99" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D99" s="71" t="s">
@@ -18319,11 +18313,11 @@
     <row r="102" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="103" spans="1:8" ht="46.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A103" s="77"/>
-      <c r="B103" s="229" t="s">
+      <c r="B103" s="241" t="s">
         <v>162</v>
       </c>
-      <c r="C103" s="200"/>
-      <c r="D103" s="201"/>
+      <c r="C103" s="237"/>
+      <c r="D103" s="242"/>
       <c r="E103" s="92" t="s">
         <v>136</v>
       </c>
@@ -18335,7 +18329,7 @@
     </row>
     <row r="104" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A104" s="77"/>
-      <c r="B104" s="232" t="s">
+      <c r="B104" s="245" t="s">
         <v>138</v>
       </c>
       <c r="C104" s="78">
@@ -18344,7 +18338,7 @@
       <c r="D104" s="79" t="s">
         <v>151</v>
       </c>
-      <c r="E104" s="269">
+      <c r="E104" s="272">
         <f>COUNTA(D14:D96)-COUNTIFS(D14:D96,0)</f>
         <v>62</v>
       </c>
@@ -18359,14 +18353,14 @@
     </row>
     <row r="105" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A105" s="77"/>
-      <c r="B105" s="233"/>
+      <c r="B105" s="246"/>
       <c r="C105" s="81">
         <v>0.6</v>
       </c>
       <c r="D105" s="82" t="s">
         <v>151</v>
       </c>
-      <c r="E105" s="212"/>
+      <c r="E105" s="273"/>
       <c r="F105" s="94">
         <f>C105*$E104</f>
         <v>37.199999999999996</v>
@@ -18378,14 +18372,14 @@
     </row>
     <row r="106" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A106" s="77"/>
-      <c r="B106" s="234"/>
+      <c r="B106" s="247"/>
       <c r="C106" s="84">
         <v>0.7</v>
       </c>
       <c r="D106" s="85" t="s">
         <v>151</v>
       </c>
-      <c r="E106" s="213"/>
+      <c r="E106" s="219"/>
       <c r="F106" s="95">
         <f>C106*$E104</f>
         <v>43.4</v>
@@ -18416,10 +18410,10 @@
       <c r="H108" s="77"/>
     </row>
     <row r="109" spans="1:8" ht="33" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A109" s="214" t="s">
+      <c r="A109" s="285" t="s">
         <v>163</v>
       </c>
-      <c r="B109" s="272"/>
+      <c r="B109" s="286"/>
       <c r="C109" s="96" t="s">
         <v>9</v>
       </c>
@@ -18440,10 +18434,10 @@
       </c>
     </row>
     <row r="110" spans="1:8" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A110" s="273" t="s">
+      <c r="A110" s="287" t="s">
         <v>164</v>
       </c>
-      <c r="B110" s="263"/>
+      <c r="B110" s="278"/>
       <c r="C110" s="98">
         <f>IF(E99&gt;=$F106,3,IF(E99&gt;=$F105,2,IF(E99&gt;=$F104,1,0)))</f>
         <v>0</v>
@@ -18470,10 +18464,10 @@
       </c>
     </row>
     <row r="111" spans="1:8" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A111" s="274" t="s">
+      <c r="A111" s="288" t="s">
         <v>165</v>
       </c>
-      <c r="B111" s="242"/>
+      <c r="B111" s="229"/>
       <c r="C111" s="100">
         <f>IF(F99&gt;=$F106,3,IF(F99&gt;=$F105,2,IF(F99&gt;=$F104,1,0)))</f>
         <v>3</v>
@@ -18500,10 +18494,10 @@
       </c>
     </row>
     <row r="112" spans="1:8" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A112" s="275" t="s">
+      <c r="A112" s="281" t="s">
         <v>166</v>
       </c>
-      <c r="B112" s="265"/>
+      <c r="B112" s="267"/>
       <c r="C112" s="62">
         <f>IF(G99&gt;=$F106,3,IF(G99&gt;=$F105,2,IF(G99&gt;=$F104,1,0)))</f>
         <v>3</v>
@@ -19429,6 +19423,13 @@
     <row r="1000" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="20">
+    <mergeCell ref="D4:E4"/>
+    <mergeCell ref="D5:E5"/>
+    <mergeCell ref="D6:E6"/>
+    <mergeCell ref="D7:E7"/>
+    <mergeCell ref="B9:B13"/>
+    <mergeCell ref="C9:C13"/>
+    <mergeCell ref="D9:D13"/>
     <mergeCell ref="A112:B112"/>
     <mergeCell ref="E9:E12"/>
     <mergeCell ref="F9:F12"/>
@@ -19442,13 +19443,6 @@
     <mergeCell ref="A109:B109"/>
     <mergeCell ref="A110:B110"/>
     <mergeCell ref="A111:B111"/>
-    <mergeCell ref="D4:E4"/>
-    <mergeCell ref="D5:E5"/>
-    <mergeCell ref="D6:E6"/>
-    <mergeCell ref="D7:E7"/>
-    <mergeCell ref="B9:B13"/>
-    <mergeCell ref="C9:C13"/>
-    <mergeCell ref="D9:D13"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup scale="28" orientation="landscape"/>
@@ -19457,7 +19451,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <tabColor rgb="FFFFFF00"/>
   </sheetPr>
@@ -19550,41 +19544,41 @@
       </c>
     </row>
     <row r="10" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B10" s="284" t="s">
+      <c r="B10" s="302" t="s">
         <v>20</v>
       </c>
-      <c r="C10" s="285" t="s">
+      <c r="C10" s="290" t="s">
         <v>169</v>
       </c>
-      <c r="D10" s="286" t="s">
+      <c r="D10" s="303" t="s">
         <v>55</v>
       </c>
-      <c r="E10" s="285" t="s">
+      <c r="E10" s="290" t="s">
         <v>170</v>
       </c>
     </row>
     <row r="11" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B11" s="212"/>
-      <c r="C11" s="212"/>
-      <c r="D11" s="212"/>
-      <c r="E11" s="212"/>
+      <c r="B11" s="273"/>
+      <c r="C11" s="273"/>
+      <c r="D11" s="273"/>
+      <c r="E11" s="273"/>
     </row>
     <row r="12" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B12" s="212"/>
-      <c r="C12" s="212"/>
-      <c r="D12" s="212"/>
-      <c r="E12" s="212"/>
+      <c r="B12" s="273"/>
+      <c r="C12" s="273"/>
+      <c r="D12" s="273"/>
+      <c r="E12" s="273"/>
     </row>
     <row r="13" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B13" s="212"/>
-      <c r="C13" s="212"/>
-      <c r="D13" s="212"/>
-      <c r="E13" s="287"/>
+      <c r="B13" s="273"/>
+      <c r="C13" s="273"/>
+      <c r="D13" s="273"/>
+      <c r="E13" s="291"/>
     </row>
     <row r="14" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B14" s="213"/>
-      <c r="C14" s="213"/>
-      <c r="D14" s="213"/>
+      <c r="B14" s="219"/>
+      <c r="C14" s="219"/>
+      <c r="D14" s="219"/>
       <c r="E14" s="105">
         <v>5</v>
       </c>
@@ -20381,57 +20375,57 @@
     </row>
     <row r="84" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="85" spans="1:7" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A85" s="288" t="s">
+      <c r="A85" s="292" t="s">
         <v>175</v>
       </c>
-      <c r="B85" s="200"/>
-      <c r="C85" s="200"/>
-      <c r="D85" s="201"/>
+      <c r="B85" s="237"/>
+      <c r="C85" s="237"/>
+      <c r="D85" s="242"/>
       <c r="E85" s="112" t="s">
         <v>137</v>
       </c>
     </row>
     <row r="86" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A86" s="289" t="s">
+      <c r="A86" s="293" t="s">
         <v>138</v>
       </c>
-      <c r="B86" s="290" t="s">
+      <c r="B86" s="294" t="s">
         <v>176</v>
       </c>
-      <c r="C86" s="291"/>
-      <c r="D86" s="268"/>
+      <c r="C86" s="295"/>
+      <c r="D86" s="271"/>
       <c r="E86" s="113">
         <v>1</v>
       </c>
     </row>
     <row r="87" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A87" s="233"/>
-      <c r="B87" s="278" t="s">
+      <c r="A87" s="246"/>
+      <c r="B87" s="296" t="s">
         <v>177</v>
       </c>
-      <c r="C87" s="279"/>
-      <c r="D87" s="255"/>
+      <c r="C87" s="297"/>
+      <c r="D87" s="257"/>
       <c r="E87" s="114">
         <v>2</v>
       </c>
     </row>
     <row r="88" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A88" s="234"/>
-      <c r="B88" s="280" t="s">
+      <c r="A88" s="247"/>
+      <c r="B88" s="298" t="s">
         <v>178</v>
       </c>
-      <c r="C88" s="281"/>
-      <c r="D88" s="227"/>
+      <c r="C88" s="299"/>
+      <c r="D88" s="239"/>
       <c r="E88" s="115">
         <v>3</v>
       </c>
     </row>
     <row r="89" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="90" spans="1:7" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A90" s="282" t="s">
+      <c r="A90" s="300" t="s">
         <v>163</v>
       </c>
-      <c r="B90" s="272"/>
+      <c r="B90" s="286"/>
       <c r="C90" s="116" t="s">
         <v>9</v>
       </c>
@@ -20449,10 +20443,10 @@
       </c>
     </row>
     <row r="91" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A91" s="283" t="s">
+      <c r="A91" s="301" t="s">
         <v>179</v>
       </c>
-      <c r="B91" s="263"/>
+      <c r="B91" s="278"/>
       <c r="C91" s="118">
         <f>IF(E81&gt;=80,3,IF(E81&gt;=65,2,IF(E81&gt;=40,1,0)))</f>
         <v>0</v>
@@ -21394,17 +21388,17 @@
     <row r="1000" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="11">
+    <mergeCell ref="A90:B90"/>
+    <mergeCell ref="A91:B91"/>
+    <mergeCell ref="B10:B14"/>
+    <mergeCell ref="C10:C14"/>
+    <mergeCell ref="D10:D14"/>
     <mergeCell ref="E10:E13"/>
     <mergeCell ref="A85:D85"/>
     <mergeCell ref="A86:A88"/>
     <mergeCell ref="B86:D86"/>
     <mergeCell ref="B87:D87"/>
     <mergeCell ref="B88:D88"/>
-    <mergeCell ref="A90:B90"/>
-    <mergeCell ref="A91:B91"/>
-    <mergeCell ref="B10:B14"/>
-    <mergeCell ref="C10:C14"/>
-    <mergeCell ref="D10:D14"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup orientation="portrait"/>
@@ -21412,7 +21406,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="B1:P1000"/>
   <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
@@ -21469,34 +21463,34 @@
       <c r="P5" s="15"/>
     </row>
     <row r="6" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B6" s="211" t="s">
+      <c r="B6" s="305" t="s">
         <v>20</v>
       </c>
-      <c r="C6" s="193" t="s">
+      <c r="C6" s="306" t="s">
         <v>21</v>
       </c>
-      <c r="D6" s="194"/>
-      <c r="E6" s="214" t="s">
+      <c r="D6" s="249"/>
+      <c r="E6" s="285" t="s">
         <v>22</v>
       </c>
-      <c r="F6" s="200"/>
-      <c r="G6" s="200"/>
-      <c r="H6" s="200"/>
-      <c r="I6" s="200"/>
-      <c r="J6" s="200"/>
-      <c r="K6" s="200"/>
-      <c r="L6" s="200"/>
-      <c r="M6" s="200"/>
-      <c r="N6" s="201"/>
-      <c r="O6" s="214" t="s">
+      <c r="F6" s="237"/>
+      <c r="G6" s="237"/>
+      <c r="H6" s="237"/>
+      <c r="I6" s="237"/>
+      <c r="J6" s="237"/>
+      <c r="K6" s="237"/>
+      <c r="L6" s="237"/>
+      <c r="M6" s="237"/>
+      <c r="N6" s="242"/>
+      <c r="O6" s="285" t="s">
         <v>23</v>
       </c>
-      <c r="P6" s="201"/>
+      <c r="P6" s="242"/>
     </row>
     <row r="7" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B7" s="212"/>
-      <c r="C7" s="195"/>
-      <c r="D7" s="196"/>
+      <c r="B7" s="273"/>
+      <c r="C7" s="250"/>
+      <c r="D7" s="251"/>
       <c r="E7" s="17" t="s">
         <v>24</v>
       </c>
@@ -21535,9 +21529,9 @@
       </c>
     </row>
     <row r="8" spans="2:16" ht="62.25" x14ac:dyDescent="0.25">
-      <c r="B8" s="213"/>
-      <c r="C8" s="197"/>
-      <c r="D8" s="198"/>
+      <c r="B8" s="219"/>
+      <c r="C8" s="252"/>
+      <c r="D8" s="253"/>
       <c r="E8" s="18" t="s">
         <v>188</v>
       </c>
@@ -21858,11 +21852,11 @@
       </c>
     </row>
     <row r="15" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B15" s="292" t="s">
+      <c r="B15" s="307" t="s">
         <v>207</v>
       </c>
-      <c r="C15" s="200"/>
-      <c r="D15" s="201"/>
+      <c r="C15" s="237"/>
+      <c r="D15" s="242"/>
       <c r="E15" s="125">
         <f t="shared" ref="E15:P15" si="0">ROUNDUP(AVERAGE(E9:E14),2)</f>
         <v>3</v>
@@ -21913,11 +21907,11 @@
       </c>
     </row>
     <row r="16" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B16" s="293" t="s">
+      <c r="B16" s="304" t="s">
         <v>208</v>
       </c>
-      <c r="C16" s="200"/>
-      <c r="D16" s="201"/>
+      <c r="C16" s="237"/>
+      <c r="D16" s="242"/>
       <c r="E16" s="126">
         <f t="shared" ref="E16:P16" si="1">ROUNDUP((E15*2.66)/3,2)</f>
         <v>2.66</v>
@@ -21968,11 +21962,11 @@
       </c>
     </row>
     <row r="17" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B17" s="293" t="s">
+      <c r="B17" s="304" t="s">
         <v>209</v>
       </c>
-      <c r="C17" s="200"/>
-      <c r="D17" s="201"/>
+      <c r="C17" s="237"/>
+      <c r="D17" s="242"/>
       <c r="E17" s="126">
         <f t="shared" ref="E17:P17" si="2">ROUNDUP((E16/3)*100,2)</f>
         <v>88.67</v>
@@ -23004,13 +22998,13 @@
     <row r="1000" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="7">
+    <mergeCell ref="O6:P6"/>
+    <mergeCell ref="B15:D15"/>
     <mergeCell ref="B16:D16"/>
     <mergeCell ref="B17:D17"/>
     <mergeCell ref="B6:B8"/>
     <mergeCell ref="C6:D8"/>
     <mergeCell ref="E6:N6"/>
-    <mergeCell ref="O6:P6"/>
-    <mergeCell ref="B15:D15"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>
@@ -23018,7 +23012,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <tabColor rgb="FFFFFF00"/>
   </sheetPr>
@@ -23259,16 +23253,16 @@
     <row r="8" spans="1:26" ht="21" x14ac:dyDescent="0.25">
       <c r="A8" s="15"/>
       <c r="B8" s="15"/>
-      <c r="C8" s="294" t="s">
+      <c r="C8" s="314" t="s">
         <v>211</v>
       </c>
-      <c r="D8" s="200"/>
-      <c r="E8" s="200"/>
-      <c r="F8" s="200"/>
-      <c r="G8" s="200"/>
-      <c r="H8" s="200"/>
-      <c r="I8" s="200"/>
-      <c r="J8" s="201"/>
+      <c r="D8" s="237"/>
+      <c r="E8" s="237"/>
+      <c r="F8" s="237"/>
+      <c r="G8" s="237"/>
+      <c r="H8" s="237"/>
+      <c r="I8" s="237"/>
+      <c r="J8" s="242"/>
       <c r="K8" s="15"/>
       <c r="L8" s="15"/>
       <c r="M8" s="15"/>
@@ -23289,18 +23283,18 @@
     <row r="9" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A9" s="15"/>
       <c r="B9" s="15"/>
-      <c r="C9" s="295" t="s">
+      <c r="C9" s="315" t="s">
         <v>212</v>
       </c>
-      <c r="D9" s="200"/>
-      <c r="E9" s="200"/>
-      <c r="F9" s="200"/>
-      <c r="G9" s="200"/>
-      <c r="H9" s="201"/>
-      <c r="I9" s="296" t="s">
+      <c r="D9" s="237"/>
+      <c r="E9" s="237"/>
+      <c r="F9" s="237"/>
+      <c r="G9" s="237"/>
+      <c r="H9" s="242"/>
+      <c r="I9" s="316" t="s">
         <v>213</v>
       </c>
-      <c r="J9" s="194"/>
+      <c r="J9" s="249"/>
       <c r="K9" s="15"/>
       <c r="L9" s="15"/>
       <c r="M9" s="15"/>
@@ -23321,20 +23315,20 @@
     <row r="10" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A10" s="15"/>
       <c r="B10" s="15"/>
-      <c r="C10" s="297" t="s">
+      <c r="C10" s="317" t="s">
         <v>214</v>
       </c>
-      <c r="D10" s="298" t="s">
+      <c r="D10" s="318" t="s">
         <v>215</v>
       </c>
-      <c r="E10" s="299"/>
-      <c r="F10" s="299"/>
-      <c r="G10" s="198"/>
+      <c r="E10" s="319"/>
+      <c r="F10" s="319"/>
+      <c r="G10" s="253"/>
       <c r="H10" s="128" t="s">
         <v>216</v>
       </c>
-      <c r="I10" s="197"/>
-      <c r="J10" s="198"/>
+      <c r="I10" s="252"/>
+      <c r="J10" s="253"/>
       <c r="K10" s="15"/>
       <c r="L10" s="15"/>
       <c r="M10" s="15"/>
@@ -23355,7 +23349,7 @@
     <row r="11" spans="1:26" ht="45.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="15"/>
       <c r="B11" s="15"/>
-      <c r="C11" s="213"/>
+      <c r="C11" s="219"/>
       <c r="D11" s="129" t="s">
         <v>217</v>
       </c>
@@ -23371,10 +23365,10 @@
       <c r="H11" s="132" t="s">
         <v>220</v>
       </c>
-      <c r="I11" s="300" t="s">
+      <c r="I11" s="320" t="s">
         <v>221</v>
       </c>
-      <c r="J11" s="201"/>
+      <c r="J11" s="242"/>
       <c r="K11" s="15"/>
       <c r="L11" s="15"/>
       <c r="M11" s="15"/>
@@ -23418,11 +23412,11 @@
         <f>'CO_attainment for FA-TH ESE'!C110</f>
         <v>3</v>
       </c>
-      <c r="I12" s="301">
+      <c r="I12" s="310">
         <f>'CO_attainment for Indirect'!C91</f>
         <v>0</v>
       </c>
-      <c r="J12" s="268"/>
+      <c r="J12" s="271"/>
       <c r="K12" s="15"/>
       <c r="L12" s="15"/>
       <c r="M12" s="15"/>
@@ -23466,11 +23460,11 @@
         <f t="shared" ref="H13:H17" si="3">$H12</f>
         <v>3</v>
       </c>
-      <c r="I13" s="305">
+      <c r="I13" s="309">
         <f t="shared" ref="I13:I17" si="4">$I12</f>
         <v>0</v>
       </c>
-      <c r="J13" s="255"/>
+      <c r="J13" s="257"/>
       <c r="K13" s="15"/>
       <c r="L13" s="15"/>
       <c r="M13" s="15"/>
@@ -23514,11 +23508,11 @@
         <f t="shared" si="3"/>
         <v>3</v>
       </c>
-      <c r="I14" s="305">
+      <c r="I14" s="309">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="J14" s="255"/>
+      <c r="J14" s="257"/>
       <c r="K14" s="15"/>
       <c r="L14" s="15"/>
       <c r="M14" s="15"/>
@@ -23562,11 +23556,11 @@
         <f t="shared" si="3"/>
         <v>3</v>
       </c>
-      <c r="I15" s="305">
+      <c r="I15" s="309">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="J15" s="255"/>
+      <c r="J15" s="257"/>
       <c r="K15" s="15"/>
       <c r="L15" s="15"/>
       <c r="M15" s="15"/>
@@ -23610,11 +23604,11 @@
         <f t="shared" si="3"/>
         <v>3</v>
       </c>
-      <c r="I16" s="305">
+      <c r="I16" s="309">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="J16" s="255"/>
+      <c r="J16" s="257"/>
       <c r="K16" s="15"/>
       <c r="L16" s="15"/>
       <c r="M16" s="15"/>
@@ -23658,11 +23652,11 @@
         <f t="shared" si="3"/>
         <v>3</v>
       </c>
-      <c r="I17" s="305">
+      <c r="I17" s="309">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="J17" s="255"/>
+      <c r="J17" s="257"/>
       <c r="K17" s="15"/>
       <c r="L17" s="15"/>
       <c r="M17" s="15"/>
@@ -23706,11 +23700,11 @@
         <f t="shared" si="5"/>
         <v>3</v>
       </c>
-      <c r="I18" s="301">
+      <c r="I18" s="310">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="J18" s="268"/>
+      <c r="J18" s="271"/>
       <c r="K18" s="15"/>
       <c r="L18" s="15"/>
       <c r="M18" s="15"/>
@@ -23749,10 +23743,10 @@
       <c r="H19" s="146">
         <v>60</v>
       </c>
-      <c r="I19" s="306">
+      <c r="I19" s="311">
         <v>100</v>
       </c>
-      <c r="J19" s="242"/>
+      <c r="J19" s="229"/>
       <c r="K19" s="15"/>
       <c r="L19" s="15"/>
       <c r="M19" s="15"/>
@@ -23796,11 +23790,11 @@
         <f t="shared" si="6"/>
         <v>1.8</v>
       </c>
-      <c r="I20" s="302">
+      <c r="I20" s="312">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="J20" s="227"/>
+      <c r="J20" s="239"/>
       <c r="K20" s="15"/>
       <c r="L20" s="15"/>
       <c r="M20" s="15"/>
@@ -23821,13 +23815,13 @@
     <row r="21" spans="1:26" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="15"/>
       <c r="B21" s="15"/>
-      <c r="C21" s="303" t="s">
+      <c r="C21" s="313" t="s">
         <v>225</v>
       </c>
-      <c r="D21" s="200"/>
-      <c r="E21" s="200"/>
-      <c r="F21" s="200"/>
-      <c r="G21" s="201"/>
+      <c r="D21" s="237"/>
+      <c r="E21" s="237"/>
+      <c r="F21" s="237"/>
+      <c r="G21" s="242"/>
       <c r="H21" s="148">
         <f>SUM(D20:H20)</f>
         <v>2.4</v>
@@ -23859,13 +23853,13 @@
     <row r="22" spans="1:26" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="15"/>
       <c r="B22" s="15"/>
-      <c r="C22" s="303" t="s">
+      <c r="C22" s="313" t="s">
         <v>227</v>
       </c>
-      <c r="D22" s="200"/>
-      <c r="E22" s="200"/>
-      <c r="F22" s="200"/>
-      <c r="G22" s="201"/>
+      <c r="D22" s="237"/>
+      <c r="E22" s="237"/>
+      <c r="F22" s="237"/>
+      <c r="G22" s="242"/>
       <c r="H22" s="150">
         <v>0.8</v>
       </c>
@@ -23895,13 +23889,13 @@
     <row r="23" spans="1:26" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="15"/>
       <c r="B23" s="15"/>
-      <c r="C23" s="303" t="s">
+      <c r="C23" s="313" t="s">
         <v>229</v>
       </c>
-      <c r="D23" s="200"/>
-      <c r="E23" s="200"/>
-      <c r="F23" s="200"/>
-      <c r="G23" s="201"/>
+      <c r="D23" s="237"/>
+      <c r="E23" s="237"/>
+      <c r="F23" s="237"/>
+      <c r="G23" s="242"/>
       <c r="H23" s="148">
         <f>0.8*H21</f>
         <v>1.92</v>
@@ -23933,14 +23927,14 @@
     <row r="24" spans="1:26" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="15"/>
       <c r="B24" s="15"/>
-      <c r="C24" s="304" t="s">
+      <c r="C24" s="308" t="s">
         <v>231</v>
       </c>
-      <c r="D24" s="200"/>
-      <c r="E24" s="200"/>
-      <c r="F24" s="200"/>
-      <c r="G24" s="200"/>
-      <c r="H24" s="201"/>
+      <c r="D24" s="237"/>
+      <c r="E24" s="237"/>
+      <c r="F24" s="237"/>
+      <c r="G24" s="237"/>
+      <c r="H24" s="242"/>
       <c r="I24" s="152">
         <f>ROUNDUP(H23+J23,2)</f>
         <v>1.92</v>
@@ -30534,6 +30528,17 @@
     <row r="1000" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="19">
+    <mergeCell ref="C8:J8"/>
+    <mergeCell ref="C9:H9"/>
+    <mergeCell ref="I9:J10"/>
+    <mergeCell ref="C10:C11"/>
+    <mergeCell ref="D10:G10"/>
+    <mergeCell ref="I11:J11"/>
+    <mergeCell ref="I12:J12"/>
+    <mergeCell ref="I20:J20"/>
+    <mergeCell ref="C21:G21"/>
+    <mergeCell ref="C22:G22"/>
+    <mergeCell ref="C23:G23"/>
     <mergeCell ref="C24:H24"/>
     <mergeCell ref="I13:J13"/>
     <mergeCell ref="I14:J14"/>
@@ -30542,17 +30547,6 @@
     <mergeCell ref="I17:J17"/>
     <mergeCell ref="I18:J18"/>
     <mergeCell ref="I19:J19"/>
-    <mergeCell ref="I12:J12"/>
-    <mergeCell ref="I20:J20"/>
-    <mergeCell ref="C21:G21"/>
-    <mergeCell ref="C22:G22"/>
-    <mergeCell ref="C23:G23"/>
-    <mergeCell ref="C8:J8"/>
-    <mergeCell ref="C9:H9"/>
-    <mergeCell ref="I9:J10"/>
-    <mergeCell ref="C10:C11"/>
-    <mergeCell ref="D10:G10"/>
-    <mergeCell ref="I11:J11"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup orientation="portrait"/>
@@ -30560,7 +30554,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <tabColor rgb="FFFFFF00"/>
   </sheetPr>
@@ -30802,15 +30796,15 @@
     <row r="8" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A8" s="15"/>
       <c r="B8" s="27"/>
-      <c r="C8" s="307" t="s">
+      <c r="C8" s="335" t="s">
         <v>234</v>
       </c>
-      <c r="D8" s="308"/>
-      <c r="E8" s="310" t="s">
+      <c r="D8" s="336"/>
+      <c r="E8" s="338" t="s">
         <v>235</v>
       </c>
-      <c r="F8" s="291"/>
-      <c r="G8" s="263"/>
+      <c r="F8" s="295"/>
+      <c r="G8" s="278"/>
       <c r="H8" s="154" t="s">
         <v>159</v>
       </c>
@@ -30820,7 +30814,7 @@
       <c r="J8" s="154" t="s">
         <v>236</v>
       </c>
-      <c r="K8" s="311" t="s">
+      <c r="K8" s="339" t="s">
         <v>237</v>
       </c>
       <c r="L8" s="15"/>
@@ -30842,8 +30836,8 @@
     <row r="9" spans="1:26" ht="30" x14ac:dyDescent="0.25">
       <c r="A9" s="15"/>
       <c r="B9" s="27"/>
-      <c r="C9" s="197"/>
-      <c r="D9" s="309"/>
+      <c r="C9" s="252"/>
+      <c r="D9" s="337"/>
       <c r="E9" s="155" t="s">
         <v>238</v>
       </c>
@@ -30862,7 +30856,7 @@
       <c r="J9" s="156" t="s">
         <v>220</v>
       </c>
-      <c r="K9" s="312"/>
+      <c r="K9" s="340"/>
       <c r="L9" s="15"/>
       <c r="M9" s="15"/>
       <c r="N9" s="15"/>
@@ -30882,14 +30876,14 @@
     <row r="10" spans="1:26" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="15"/>
       <c r="B10" s="27"/>
-      <c r="C10" s="313" t="s">
+      <c r="C10" s="341" t="s">
         <v>242</v>
       </c>
-      <c r="D10" s="263"/>
-      <c r="E10" s="314">
+      <c r="D10" s="278"/>
+      <c r="E10" s="342">
         <v>20</v>
       </c>
-      <c r="F10" s="263"/>
+      <c r="F10" s="278"/>
       <c r="G10" s="157">
         <v>10</v>
       </c>
@@ -30925,15 +30919,15 @@
     <row r="11" spans="1:26" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="15"/>
       <c r="B11" s="27"/>
-      <c r="C11" s="315" t="s">
+      <c r="C11" s="328" t="s">
         <v>243</v>
       </c>
-      <c r="D11" s="265"/>
-      <c r="E11" s="316">
+      <c r="D11" s="267"/>
+      <c r="E11" s="329">
         <f>(E10/$K10)*100</f>
         <v>13.333333333333334</v>
       </c>
-      <c r="F11" s="265"/>
+      <c r="F11" s="267"/>
       <c r="G11" s="158">
         <f t="shared" ref="G11:J11" si="1">(G10/$K10)*100</f>
         <v>6.666666666666667</v>
@@ -31057,16 +31051,16 @@
     <row r="15" spans="1:26" ht="21" x14ac:dyDescent="0.25">
       <c r="A15" s="15"/>
       <c r="B15" s="15"/>
-      <c r="C15" s="317" t="s">
+      <c r="C15" s="330" t="s">
         <v>211</v>
       </c>
-      <c r="D15" s="200"/>
-      <c r="E15" s="200"/>
-      <c r="F15" s="200"/>
-      <c r="G15" s="200"/>
-      <c r="H15" s="200"/>
-      <c r="I15" s="200"/>
-      <c r="J15" s="201"/>
+      <c r="D15" s="237"/>
+      <c r="E15" s="237"/>
+      <c r="F15" s="237"/>
+      <c r="G15" s="237"/>
+      <c r="H15" s="237"/>
+      <c r="I15" s="237"/>
+      <c r="J15" s="242"/>
       <c r="K15" s="15"/>
       <c r="L15" s="15"/>
       <c r="M15" s="15"/>
@@ -31087,16 +31081,16 @@
     <row r="16" spans="1:26" ht="21" x14ac:dyDescent="0.25">
       <c r="A16" s="15"/>
       <c r="B16" s="15"/>
-      <c r="C16" s="318" t="s">
+      <c r="C16" s="331" t="s">
         <v>212</v>
       </c>
-      <c r="D16" s="200"/>
-      <c r="E16" s="200"/>
-      <c r="F16" s="200"/>
-      <c r="G16" s="200"/>
-      <c r="H16" s="201"/>
-      <c r="I16" s="319"/>
-      <c r="J16" s="194"/>
+      <c r="D16" s="237"/>
+      <c r="E16" s="237"/>
+      <c r="F16" s="237"/>
+      <c r="G16" s="237"/>
+      <c r="H16" s="242"/>
+      <c r="I16" s="332"/>
+      <c r="J16" s="249"/>
       <c r="K16" s="15"/>
       <c r="L16" s="15"/>
       <c r="M16" s="15"/>
@@ -31117,7 +31111,7 @@
     <row r="17" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A17" s="15"/>
       <c r="B17" s="15"/>
-      <c r="C17" s="320" t="s">
+      <c r="C17" s="333" t="s">
         <v>244</v>
       </c>
       <c r="D17" s="160"/>
@@ -31129,8 +31123,8 @@
       <c r="H17" s="164" t="s">
         <v>216</v>
       </c>
-      <c r="I17" s="197"/>
-      <c r="J17" s="198"/>
+      <c r="I17" s="252"/>
+      <c r="J17" s="253"/>
       <c r="K17" s="15"/>
       <c r="L17" s="15"/>
       <c r="M17" s="15"/>
@@ -31151,7 +31145,7 @@
     <row r="18" spans="1:26" ht="45.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="15"/>
       <c r="B18" s="15"/>
-      <c r="C18" s="213"/>
+      <c r="C18" s="219"/>
       <c r="D18" s="165" t="s">
         <v>217</v>
       </c>
@@ -31167,8 +31161,8 @@
       <c r="H18" s="168" t="s">
         <v>220</v>
       </c>
-      <c r="I18" s="321"/>
-      <c r="J18" s="201"/>
+      <c r="I18" s="334"/>
+      <c r="J18" s="242"/>
       <c r="K18" s="15"/>
       <c r="L18" s="15"/>
       <c r="M18" s="15"/>
@@ -31212,8 +31206,8 @@
         <f>'CO_attainment for FA-TH ESE'!C110</f>
         <v>3</v>
       </c>
-      <c r="I19" s="322"/>
-      <c r="J19" s="268"/>
+      <c r="I19" s="324"/>
+      <c r="J19" s="271"/>
       <c r="K19" s="15"/>
       <c r="L19" s="15"/>
       <c r="M19" s="15"/>
@@ -31258,7 +31252,7 @@
         <v>3</v>
       </c>
       <c r="I20" s="323"/>
-      <c r="J20" s="255"/>
+      <c r="J20" s="257"/>
       <c r="K20" s="15"/>
       <c r="L20" s="15"/>
       <c r="M20" s="15"/>
@@ -31303,7 +31297,7 @@
         <v>3</v>
       </c>
       <c r="I21" s="323"/>
-      <c r="J21" s="255"/>
+      <c r="J21" s="257"/>
       <c r="K21" s="15"/>
       <c r="L21" s="15"/>
       <c r="M21" s="15"/>
@@ -31348,7 +31342,7 @@
         <v>3</v>
       </c>
       <c r="I22" s="323"/>
-      <c r="J22" s="255"/>
+      <c r="J22" s="257"/>
       <c r="K22" s="15"/>
       <c r="L22" s="15"/>
       <c r="M22" s="15"/>
@@ -31393,7 +31387,7 @@
         <v>3</v>
       </c>
       <c r="I23" s="323"/>
-      <c r="J23" s="255"/>
+      <c r="J23" s="257"/>
       <c r="K23" s="15"/>
       <c r="L23" s="15"/>
       <c r="M23" s="15"/>
@@ -31438,7 +31432,7 @@
         <v>3</v>
       </c>
       <c r="I24" s="323"/>
-      <c r="J24" s="255"/>
+      <c r="J24" s="257"/>
       <c r="K24" s="15"/>
       <c r="L24" s="15"/>
       <c r="M24" s="15"/>
@@ -31482,8 +31476,8 @@
         <f t="shared" si="6"/>
         <v>3</v>
       </c>
-      <c r="I25" s="322"/>
-      <c r="J25" s="268"/>
+      <c r="I25" s="324"/>
+      <c r="J25" s="271"/>
       <c r="K25" s="15"/>
       <c r="L25" s="15"/>
       <c r="M25" s="15"/>
@@ -31527,8 +31521,8 @@
         <f t="shared" si="7"/>
         <v>46.666666666666664</v>
       </c>
-      <c r="I26" s="327"/>
-      <c r="J26" s="255"/>
+      <c r="I26" s="325"/>
+      <c r="J26" s="257"/>
       <c r="K26" s="15"/>
       <c r="L26" s="15"/>
       <c r="M26" s="15"/>
@@ -31572,8 +31566,8 @@
         <f t="shared" si="8"/>
         <v>1.4</v>
       </c>
-      <c r="I27" s="328"/>
-      <c r="J27" s="227"/>
+      <c r="I27" s="326"/>
+      <c r="J27" s="239"/>
       <c r="K27" s="15"/>
       <c r="L27" s="15"/>
       <c r="M27" s="15"/>
@@ -31594,13 +31588,13 @@
     <row r="28" spans="1:26" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="15"/>
       <c r="B28" s="15"/>
-      <c r="C28" s="324" t="s">
+      <c r="C28" s="327" t="s">
         <v>225</v>
       </c>
-      <c r="D28" s="200"/>
-      <c r="E28" s="200"/>
-      <c r="F28" s="200"/>
-      <c r="G28" s="201"/>
+      <c r="D28" s="237"/>
+      <c r="E28" s="237"/>
+      <c r="F28" s="237"/>
+      <c r="G28" s="242"/>
       <c r="H28" s="183">
         <f>SUM(D27:H27)</f>
         <v>2.4</v>
@@ -31627,13 +31621,13 @@
     <row r="29" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="15"/>
       <c r="B29" s="15"/>
-      <c r="C29" s="324" t="s">
+      <c r="C29" s="327" t="s">
         <v>227</v>
       </c>
-      <c r="D29" s="200"/>
-      <c r="E29" s="200"/>
-      <c r="F29" s="200"/>
-      <c r="G29" s="201"/>
+      <c r="D29" s="237"/>
+      <c r="E29" s="237"/>
+      <c r="F29" s="237"/>
+      <c r="G29" s="242"/>
       <c r="H29" s="186">
         <v>1</v>
       </c>
@@ -31659,13 +31653,13 @@
     <row r="30" spans="1:26" ht="62.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="15"/>
       <c r="B30" s="15"/>
-      <c r="C30" s="324" t="s">
+      <c r="C30" s="327" t="s">
         <v>229</v>
       </c>
-      <c r="D30" s="200"/>
-      <c r="E30" s="200"/>
-      <c r="F30" s="200"/>
-      <c r="G30" s="201"/>
+      <c r="D30" s="237"/>
+      <c r="E30" s="237"/>
+      <c r="F30" s="237"/>
+      <c r="G30" s="242"/>
       <c r="H30" s="183">
         <f>H29*H28</f>
         <v>2.4</v>
@@ -31692,14 +31686,14 @@
     <row r="31" spans="1:26" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="15"/>
       <c r="B31" s="15"/>
-      <c r="C31" s="325" t="s">
+      <c r="C31" s="321" t="s">
         <v>231</v>
       </c>
-      <c r="D31" s="200"/>
-      <c r="E31" s="200"/>
-      <c r="F31" s="200"/>
-      <c r="G31" s="200"/>
-      <c r="H31" s="201"/>
+      <c r="D31" s="237"/>
+      <c r="E31" s="237"/>
+      <c r="F31" s="237"/>
+      <c r="G31" s="237"/>
+      <c r="H31" s="242"/>
       <c r="I31" s="188">
         <f>H30+J30</f>
         <v>2.4</v>
@@ -31786,11 +31780,11 @@
       <c r="E34" s="15"/>
       <c r="F34" s="15"/>
       <c r="G34" s="15"/>
-      <c r="H34" s="208" t="s">
+      <c r="H34" s="207" t="s">
         <v>45</v>
       </c>
-      <c r="I34" s="206"/>
-      <c r="J34" s="206"/>
+      <c r="I34" s="208"/>
+      <c r="J34" s="208"/>
       <c r="L34" s="15"/>
       <c r="M34" s="15"/>
       <c r="N34" s="15"/>
@@ -31815,11 +31809,11 @@
       <c r="E35" s="15"/>
       <c r="F35" s="15"/>
       <c r="G35" s="15"/>
-      <c r="H35" s="326" t="s">
+      <c r="H35" s="322" t="s">
         <v>46</v>
       </c>
-      <c r="I35" s="210"/>
-      <c r="J35" s="210"/>
+      <c r="I35" s="206"/>
+      <c r="J35" s="206"/>
       <c r="K35" s="4"/>
       <c r="L35" s="4"/>
       <c r="M35" s="4"/>
@@ -38204,6 +38198,23 @@
     <row r="1000" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="27">
+    <mergeCell ref="C8:D9"/>
+    <mergeCell ref="E8:G8"/>
+    <mergeCell ref="K8:K9"/>
+    <mergeCell ref="C10:D10"/>
+    <mergeCell ref="E10:F10"/>
+    <mergeCell ref="C11:D11"/>
+    <mergeCell ref="E11:F11"/>
+    <mergeCell ref="C15:J15"/>
+    <mergeCell ref="C16:H16"/>
+    <mergeCell ref="I16:J17"/>
+    <mergeCell ref="C17:C18"/>
+    <mergeCell ref="I18:J18"/>
+    <mergeCell ref="I19:J19"/>
+    <mergeCell ref="I20:J20"/>
+    <mergeCell ref="C28:G28"/>
+    <mergeCell ref="C29:G29"/>
+    <mergeCell ref="C30:G30"/>
     <mergeCell ref="C31:H31"/>
     <mergeCell ref="H34:J34"/>
     <mergeCell ref="H35:J35"/>
@@ -38214,23 +38225,6 @@
     <mergeCell ref="I25:J25"/>
     <mergeCell ref="I26:J26"/>
     <mergeCell ref="I27:J27"/>
-    <mergeCell ref="I19:J19"/>
-    <mergeCell ref="I20:J20"/>
-    <mergeCell ref="C28:G28"/>
-    <mergeCell ref="C29:G29"/>
-    <mergeCell ref="C30:G30"/>
-    <mergeCell ref="C11:D11"/>
-    <mergeCell ref="E11:F11"/>
-    <mergeCell ref="C15:J15"/>
-    <mergeCell ref="C16:H16"/>
-    <mergeCell ref="I16:J17"/>
-    <mergeCell ref="C17:C18"/>
-    <mergeCell ref="I18:J18"/>
-    <mergeCell ref="C8:D9"/>
-    <mergeCell ref="E8:G8"/>
-    <mergeCell ref="K8:K9"/>
-    <mergeCell ref="C10:D10"/>
-    <mergeCell ref="E10:F10"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>
@@ -38241,7 +38235,7 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <tabColor rgb="FFFFFF00"/>
   </sheetPr>
@@ -38295,11 +38289,11 @@
       <c r="C2" s="28" t="s">
         <v>1</v>
       </c>
-      <c r="D2" s="241" t="str">
+      <c r="D2" s="228" t="str">
         <f>'Overall CO attainment'!D3</f>
         <v>Data Structures Using _C</v>
       </c>
-      <c r="E2" s="242"/>
+      <c r="E2" s="229"/>
       <c r="F2" s="4"/>
       <c r="G2" s="4"/>
       <c r="H2" s="4"/>
@@ -38327,11 +38321,11 @@
       <c r="C3" s="28" t="s">
         <v>3</v>
       </c>
-      <c r="D3" s="241">
+      <c r="D3" s="228">
         <f>'Overall CO attainment'!D4</f>
         <v>22317</v>
       </c>
-      <c r="E3" s="242"/>
+      <c r="E3" s="229"/>
       <c r="F3" s="4"/>
       <c r="G3" s="4"/>
       <c r="H3" s="4"/>
@@ -38359,11 +38353,11 @@
       <c r="C4" s="28" t="s">
         <v>4</v>
       </c>
-      <c r="D4" s="241" t="str">
+      <c r="D4" s="228" t="str">
         <f>'Overall CO attainment'!D5</f>
         <v>3rd SEM(CO3I SCHEME)</v>
       </c>
-      <c r="E4" s="242"/>
+      <c r="E4" s="229"/>
       <c r="F4" s="4"/>
       <c r="G4" s="4"/>
       <c r="H4" s="4"/>
@@ -38391,11 +38385,11 @@
       <c r="C5" s="28" t="s">
         <v>157</v>
       </c>
-      <c r="D5" s="241" t="str">
+      <c r="D5" s="228" t="str">
         <f>'Overall CO attainment'!D6</f>
         <v>2023-24</v>
       </c>
-      <c r="E5" s="242"/>
+      <c r="E5" s="229"/>
       <c r="F5" s="4"/>
       <c r="G5" s="4"/>
       <c r="H5" s="4"/>
@@ -38502,26 +38496,26 @@
     </row>
     <row r="9" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A9" s="4"/>
-      <c r="B9" s="211" t="s">
+      <c r="B9" s="305" t="s">
         <v>20</v>
       </c>
-      <c r="C9" s="193" t="s">
+      <c r="C9" s="306" t="s">
         <v>21</v>
       </c>
-      <c r="D9" s="194"/>
-      <c r="E9" s="214" t="s">
+      <c r="D9" s="249"/>
+      <c r="E9" s="285" t="s">
         <v>22</v>
       </c>
-      <c r="F9" s="200"/>
-      <c r="G9" s="200"/>
-      <c r="H9" s="200"/>
-      <c r="I9" s="200"/>
-      <c r="J9" s="200"/>
-      <c r="K9" s="201"/>
-      <c r="L9" s="214" t="s">
+      <c r="F9" s="237"/>
+      <c r="G9" s="237"/>
+      <c r="H9" s="237"/>
+      <c r="I9" s="237"/>
+      <c r="J9" s="237"/>
+      <c r="K9" s="242"/>
+      <c r="L9" s="285" t="s">
         <v>23</v>
       </c>
-      <c r="M9" s="201"/>
+      <c r="M9" s="242"/>
       <c r="N9" s="4"/>
       <c r="O9" s="4"/>
       <c r="P9" s="4"/>
@@ -38537,9 +38531,9 @@
     </row>
     <row r="10" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="4"/>
-      <c r="B10" s="212"/>
-      <c r="C10" s="195"/>
-      <c r="D10" s="196"/>
+      <c r="B10" s="273"/>
+      <c r="C10" s="250"/>
+      <c r="D10" s="251"/>
       <c r="E10" s="17" t="s">
         <v>24</v>
       </c>
@@ -38582,9 +38576,9 @@
     </row>
     <row r="11" spans="1:25" ht="119.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="4"/>
-      <c r="B11" s="213"/>
-      <c r="C11" s="197"/>
-      <c r="D11" s="198"/>
+      <c r="B11" s="219"/>
+      <c r="C11" s="252"/>
+      <c r="D11" s="253"/>
       <c r="E11" s="18" t="s">
         <v>33</v>
       </c>
@@ -38939,11 +38933,11 @@
     </row>
     <row r="17" spans="1:25" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="4"/>
-      <c r="B17" s="199" t="s">
+      <c r="B17" s="343" t="s">
         <v>247</v>
       </c>
-      <c r="C17" s="200"/>
-      <c r="D17" s="201"/>
+      <c r="C17" s="237"/>
+      <c r="D17" s="242"/>
       <c r="E17" s="20">
         <f t="shared" ref="E17:M17" si="0">IFERROR(AVERAGE(E12:E16),0)</f>
         <v>3</v>
@@ -38995,11 +38989,11 @@
     </row>
     <row r="18" spans="1:25" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="4"/>
-      <c r="B18" s="202" t="s">
+      <c r="B18" s="344" t="s">
         <v>248</v>
       </c>
-      <c r="C18" s="200"/>
-      <c r="D18" s="201"/>
+      <c r="C18" s="237"/>
+      <c r="D18" s="242"/>
       <c r="E18" s="191">
         <f>E17*'Overall CO attainment'!I31/3</f>
         <v>2.4</v>
@@ -39051,11 +39045,11 @@
     </row>
     <row r="19" spans="1:25" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="4"/>
-      <c r="B19" s="293" t="s">
+      <c r="B19" s="304" t="s">
         <v>209</v>
       </c>
-      <c r="C19" s="200"/>
-      <c r="D19" s="201"/>
+      <c r="C19" s="237"/>
+      <c r="D19" s="242"/>
       <c r="E19" s="126">
         <f t="shared" ref="E19:M19" si="1">ROUNDUP((E18/3)*100,2)</f>
         <v>80</v>
@@ -39169,12 +39163,12 @@
       <c r="G22" s="4"/>
       <c r="H22" s="4"/>
       <c r="I22" s="4"/>
-      <c r="J22" s="208" t="s">
+      <c r="J22" s="207" t="s">
         <v>45</v>
       </c>
-      <c r="K22" s="206"/>
-      <c r="L22" s="206"/>
-      <c r="M22" s="206"/>
+      <c r="K22" s="208"/>
+      <c r="L22" s="208"/>
+      <c r="M22" s="208"/>
       <c r="N22" s="4"/>
       <c r="O22" s="4"/>
       <c r="P22" s="4"/>
@@ -39201,9 +39195,9 @@
       <c r="J23" s="209" t="s">
         <v>46</v>
       </c>
-      <c r="K23" s="210"/>
-      <c r="L23" s="210"/>
-      <c r="M23" s="210"/>
+      <c r="K23" s="206"/>
+      <c r="L23" s="206"/>
+      <c r="M23" s="206"/>
       <c r="N23" s="26"/>
       <c r="O23" s="26"/>
       <c r="P23" s="4"/>

</xml_diff>